<commit_message>
Doku, CSS, Use Case Diagramm, Zeitplan
</commit_message>
<xml_diff>
--- a/pa_zeitplan_vorlage.xlsx
+++ b/pa_zeitplan_vorlage.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCD16F2-3CAD-43C2-B0C3-6BE03493A565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91C9B9C-0087-4900-9FCF-4B02E68C6C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>IPERKA Phase</t>
   </si>
@@ -41,12 +41,6 @@
   </si>
   <si>
     <t>Aufwand (h)</t>
-  </si>
-  <si>
-    <t>DD</t>
-  </si>
-  <si>
-    <t>DD.MM:YYYY</t>
   </si>
   <si>
     <t>Sollzeit</t>
@@ -119,6 +113,33 @@
   </si>
   <si>
     <t>Systembeschreibung, Kurzfassung, Anleitutungm Glossar, etc. erstellen</t>
+  </si>
+  <si>
+    <t>10min</t>
+  </si>
+  <si>
+    <t>Montag</t>
+  </si>
+  <si>
+    <t>Dienstag</t>
+  </si>
+  <si>
+    <t>Mittwoch</t>
+  </si>
+  <si>
+    <t>Donnerstag</t>
+  </si>
+  <si>
+    <t>Freitag</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t>1h 30min</t>
+  </si>
+  <si>
+    <t>User Storys aufschreiben</t>
   </si>
 </sst>
 </file>
@@ -718,7 +739,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -771,141 +792,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -916,6 +802,144 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1233,192 +1257,184 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BC51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:BC55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
-    <col min="3" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="6" width="4.33203125" customWidth="1"/>
-    <col min="7" max="11" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.33203125" customWidth="1"/>
-    <col min="13" max="13" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="4.33203125" customWidth="1"/>
-    <col min="15" max="51" width="4.33203125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="4.33203125" customWidth="1"/>
-    <col min="54" max="54" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="6" width="4.28515625" customWidth="1"/>
+    <col min="7" max="11" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.28515625" customWidth="1"/>
+    <col min="13" max="13" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.28515625" customWidth="1"/>
+    <col min="15" max="51" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="4.28515625" customWidth="1"/>
+    <col min="54" max="54" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A1" s="80" t="s">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.25">
+      <c r="A1" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="72" t="s">
+      <c r="B1" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="75" t="s">
+      <c r="C1" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="76"/>
-      <c r="E1" s="65" t="s">
+      <c r="D1" s="69"/>
+      <c r="E1" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="49"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1" s="49"/>
+      <c r="S1" s="49"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="V1" s="49"/>
+      <c r="W1" s="49"/>
+      <c r="X1" s="50"/>
+      <c r="Y1" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" s="49"/>
+      <c r="AA1" s="49"/>
+      <c r="AB1" s="50"/>
+      <c r="AC1" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD1" s="49"/>
+      <c r="AE1" s="49"/>
+      <c r="AF1" s="50"/>
+      <c r="AG1" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH1" s="49"/>
+      <c r="AI1" s="49"/>
+      <c r="AJ1" s="50"/>
+      <c r="AK1" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="AL1" s="49"/>
+      <c r="AM1" s="49"/>
+      <c r="AN1" s="50"/>
+      <c r="AO1" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="AP1" s="49"/>
+      <c r="AQ1" s="49"/>
+      <c r="AR1" s="50"/>
+      <c r="AS1" s="48"/>
+      <c r="AT1" s="49"/>
+      <c r="AU1" s="49"/>
+      <c r="AV1" s="50"/>
+      <c r="AW1" s="48"/>
+      <c r="AX1" s="49"/>
+      <c r="AY1" s="49"/>
+      <c r="AZ1" s="50"/>
+    </row>
+    <row r="2" spans="1:55" x14ac:dyDescent="0.25">
+      <c r="A2" s="59"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="55">
+        <v>44781</v>
+      </c>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="55">
+        <v>44782</v>
+      </c>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="55">
+        <v>44783</v>
+      </c>
+      <c r="N2" s="56"/>
+      <c r="O2" s="56"/>
+      <c r="P2" s="57"/>
+      <c r="Q2" s="55">
+        <v>44784</v>
+      </c>
+      <c r="R2" s="56"/>
+      <c r="S2" s="56"/>
+      <c r="T2" s="57"/>
+      <c r="U2" s="55">
+        <v>44785</v>
+      </c>
+      <c r="V2" s="56"/>
+      <c r="W2" s="56"/>
+      <c r="X2" s="57"/>
+      <c r="Y2" s="55">
+        <v>44789</v>
+      </c>
+      <c r="Z2" s="56"/>
+      <c r="AA2" s="56"/>
+      <c r="AB2" s="57"/>
+      <c r="AC2" s="55">
+        <v>44790</v>
+      </c>
+      <c r="AD2" s="56"/>
+      <c r="AE2" s="56"/>
+      <c r="AF2" s="57"/>
+      <c r="AG2" s="55">
+        <v>44791</v>
+      </c>
+      <c r="AH2" s="56"/>
+      <c r="AI2" s="56"/>
+      <c r="AJ2" s="57"/>
+      <c r="AK2" s="55">
+        <v>44792</v>
+      </c>
+      <c r="AL2" s="56"/>
+      <c r="AM2" s="56"/>
+      <c r="AN2" s="57"/>
+      <c r="AO2" s="55">
+        <v>44795</v>
+      </c>
+      <c r="AP2" s="56"/>
+      <c r="AQ2" s="56"/>
+      <c r="AR2" s="57"/>
+      <c r="AS2" s="55"/>
+      <c r="AT2" s="56"/>
+      <c r="AU2" s="56"/>
+      <c r="AV2" s="57"/>
+      <c r="AW2" s="55"/>
+      <c r="AX2" s="56"/>
+      <c r="AY2" s="56"/>
+      <c r="AZ2" s="57"/>
+    </row>
+    <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="60"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="N1" s="66"/>
-      <c r="O1" s="66"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="V1" s="66"/>
-      <c r="W1" s="66"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z1" s="66"/>
-      <c r="AA1" s="66"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD1" s="66"/>
-      <c r="AE1" s="66"/>
-      <c r="AF1" s="67"/>
-      <c r="AG1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH1" s="66"/>
-      <c r="AI1" s="66"/>
-      <c r="AJ1" s="67"/>
-      <c r="AK1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL1" s="66"/>
-      <c r="AM1" s="66"/>
-      <c r="AN1" s="67"/>
-      <c r="AO1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP1" s="66"/>
-      <c r="AQ1" s="66"/>
-      <c r="AR1" s="67"/>
-      <c r="AS1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT1" s="66"/>
-      <c r="AU1" s="66"/>
-      <c r="AV1" s="67"/>
-      <c r="AW1" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="AX1" s="66"/>
-      <c r="AY1" s="66"/>
-      <c r="AZ1" s="67"/>
-    </row>
-    <row r="2" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A2" s="81"/>
-      <c r="B2" s="73"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="69" t="s">
+      <c r="D3" s="37" t="s">
         <v>4</v>
-      </c>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="T2" s="71"/>
-      <c r="U2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="V2" s="70"/>
-      <c r="W2" s="70"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="Z2" s="70"/>
-      <c r="AA2" s="70"/>
-      <c r="AB2" s="71"/>
-      <c r="AC2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="AD2" s="70"/>
-      <c r="AE2" s="70"/>
-      <c r="AF2" s="71"/>
-      <c r="AG2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="AH2" s="70"/>
-      <c r="AI2" s="70"/>
-      <c r="AJ2" s="71"/>
-      <c r="AK2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="AL2" s="70"/>
-      <c r="AM2" s="70"/>
-      <c r="AN2" s="71"/>
-      <c r="AO2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="AP2" s="70"/>
-      <c r="AQ2" s="70"/>
-      <c r="AR2" s="71"/>
-      <c r="AS2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="AT2" s="70"/>
-      <c r="AU2" s="70"/>
-      <c r="AV2" s="71"/>
-      <c r="AW2" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="AX2" s="70"/>
-      <c r="AY2" s="70"/>
-      <c r="AZ2" s="71"/>
-    </row>
-    <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="82"/>
-      <c r="B3" s="74"/>
-      <c r="C3" s="36" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="37" t="s">
-        <v>6</v>
       </c>
       <c r="E3" s="31">
         <v>10</v>
@@ -1540,41 +1556,25 @@
       <c r="AR3" s="35">
         <v>17</v>
       </c>
-      <c r="AS3" s="31">
-        <v>10</v>
-      </c>
-      <c r="AT3" s="34">
-        <v>12</v>
-      </c>
-      <c r="AU3" s="34">
-        <v>15</v>
-      </c>
-      <c r="AV3" s="35">
-        <v>17</v>
-      </c>
-      <c r="AW3" s="31">
-        <v>10</v>
-      </c>
-      <c r="AX3" s="34">
-        <v>12</v>
-      </c>
-      <c r="AY3" s="34">
-        <v>15</v>
-      </c>
-      <c r="AZ3" s="35">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AS3" s="31"/>
+      <c r="AT3" s="34"/>
+      <c r="AU3" s="34"/>
+      <c r="AV3" s="35"/>
+      <c r="AW3" s="31"/>
+      <c r="AX3" s="34"/>
+      <c r="AY3" s="34"/>
+      <c r="AZ3" s="35"/>
+    </row>
+    <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="39" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="84"/>
-      <c r="G4" s="84"/>
+      <c r="B4" s="72" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="53"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
       <c r="H4" s="33"/>
       <c r="I4" s="30"/>
       <c r="J4" s="32"/>
@@ -1621,18 +1621,18 @@
       <c r="AY4" s="32"/>
       <c r="AZ4" s="33"/>
       <c r="BB4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BC4" s="2"/>
     </row>
-    <row r="5" spans="1:55" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="54"/>
-      <c r="C5" s="56"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="85"/>
-      <c r="F5" s="86"/>
-      <c r="G5" s="86"/>
+      <c r="B5" s="86"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="24"/>
       <c r="I5" s="20"/>
       <c r="J5" s="21"/>
@@ -1679,18 +1679,18 @@
       <c r="AY5" s="21"/>
       <c r="AZ5" s="24"/>
       <c r="BB5" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BC5" s="3"/>
     </row>
-    <row r="6" spans="1:55" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="59"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="87"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="88"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
       <c r="I6" s="11"/>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
@@ -1726,18 +1726,18 @@
       <c r="AY6" s="12"/>
       <c r="AZ6" s="13"/>
       <c r="BB6" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="BC6" s="25"/>
     </row>
-    <row r="7" spans="1:55" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="56"/>
-      <c r="D7" s="58"/>
-      <c r="E7" s="89"/>
-      <c r="F7" s="90"/>
-      <c r="G7" s="90"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="85"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="45"/>
       <c r="H7" s="16"/>
       <c r="I7" s="14"/>
       <c r="J7" s="15"/>
@@ -1784,22 +1784,26 @@
       <c r="AY7" s="15"/>
       <c r="AZ7" s="16"/>
       <c r="BB7" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="BC7" s="27"/>
     </row>
-    <row r="8" spans="1:55" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="42" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="45" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="47"/>
-      <c r="D8" s="63"/>
-      <c r="E8" s="91"/>
-      <c r="F8" s="92"/>
-      <c r="G8" s="92"/>
+    <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="61" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="80" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="91" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="46"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
       <c r="H8" s="10"/>
       <c r="I8" s="28"/>
       <c r="J8" s="9"/>
@@ -1846,18 +1850,18 @@
       <c r="AY8" s="9"/>
       <c r="AZ8" s="10"/>
       <c r="BB8" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="BC8" s="26"/>
     </row>
-    <row r="9" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A9" s="43"/>
-      <c r="B9" s="46"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="64"/>
-      <c r="E9" s="87"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
+    <row r="9" spans="1:55" x14ac:dyDescent="0.25">
+      <c r="A9" s="62"/>
+      <c r="B9" s="52"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="92"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
       <c r="H9" s="13"/>
       <c r="I9" s="11"/>
       <c r="J9" s="12"/>
@@ -1904,16 +1908,20 @@
       <c r="AY9" s="12"/>
       <c r="AZ9" s="13"/>
     </row>
-    <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="43"/>
-      <c r="B10" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="55"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="87"/>
-      <c r="F10" s="88"/>
-      <c r="G10" s="88"/>
+    <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="62"/>
+      <c r="B10" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="42"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
       <c r="H10" s="13"/>
       <c r="I10" s="11"/>
       <c r="J10" s="12"/>
@@ -1960,14 +1968,14 @@
       <c r="AY10" s="12"/>
       <c r="AZ10" s="13"/>
     </row>
-    <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="43"/>
-      <c r="B11" s="46"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="87"/>
-      <c r="F11" s="88"/>
-      <c r="G11" s="88"/>
+    <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="62"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="54"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
       <c r="H11" s="13"/>
       <c r="I11" s="11"/>
       <c r="J11" s="12"/>
@@ -2014,182 +2022,180 @@
       <c r="AY11" s="12"/>
       <c r="AZ11" s="13"/>
     </row>
-    <row r="12" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+    <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="62"/>
+      <c r="B12" s="52" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="53"/>
+      <c r="D12" s="53"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
       <c r="H12" s="13"/>
-      <c r="I12" s="20"/>
+      <c r="I12" s="11"/>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
       <c r="L12" s="13"/>
-      <c r="M12" s="20"/>
+      <c r="M12" s="11"/>
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
       <c r="P12" s="13"/>
-      <c r="Q12" s="20"/>
+      <c r="Q12" s="11"/>
       <c r="R12" s="12"/>
       <c r="S12" s="12"/>
       <c r="T12" s="13"/>
-      <c r="U12" s="20"/>
+      <c r="U12" s="11"/>
       <c r="V12" s="12"/>
       <c r="W12" s="12"/>
       <c r="X12" s="13"/>
-      <c r="Y12" s="20"/>
+      <c r="Y12" s="11"/>
       <c r="Z12" s="12"/>
       <c r="AA12" s="12"/>
       <c r="AB12" s="13"/>
-      <c r="AC12" s="20"/>
+      <c r="AC12" s="11"/>
       <c r="AD12" s="12"/>
       <c r="AE12" s="12"/>
       <c r="AF12" s="13"/>
-      <c r="AG12" s="20"/>
+      <c r="AG12" s="11"/>
       <c r="AH12" s="12"/>
       <c r="AI12" s="12"/>
       <c r="AJ12" s="13"/>
-      <c r="AK12" s="20"/>
+      <c r="AK12" s="11"/>
       <c r="AL12" s="12"/>
       <c r="AM12" s="12"/>
       <c r="AN12" s="13"/>
-      <c r="AO12" s="20"/>
+      <c r="AO12" s="11"/>
       <c r="AP12" s="12"/>
       <c r="AQ12" s="12"/>
       <c r="AR12" s="13"/>
-      <c r="AS12" s="20"/>
+      <c r="AS12" s="11"/>
       <c r="AT12" s="12"/>
       <c r="AU12" s="12"/>
       <c r="AV12" s="13"/>
-      <c r="AW12" s="20"/>
+      <c r="AW12" s="11"/>
       <c r="AX12" s="12"/>
       <c r="AY12" s="12"/>
       <c r="AZ12" s="13"/>
     </row>
-    <row r="13" spans="1:55" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="44"/>
-      <c r="B13" s="50"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="18"/>
-      <c r="P13" s="19"/>
-      <c r="Q13" s="17"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="18"/>
-      <c r="T13" s="19"/>
-      <c r="U13" s="17"/>
-      <c r="V13" s="18"/>
-      <c r="W13" s="18"/>
-      <c r="X13" s="19"/>
-      <c r="Y13" s="17"/>
-      <c r="Z13" s="18"/>
-      <c r="AA13" s="18"/>
-      <c r="AB13" s="19"/>
-      <c r="AC13" s="17"/>
-      <c r="AD13" s="18"/>
-      <c r="AE13" s="18"/>
-      <c r="AF13" s="19"/>
-      <c r="AG13" s="17"/>
-      <c r="AH13" s="18"/>
-      <c r="AI13" s="18"/>
-      <c r="AJ13" s="19"/>
-      <c r="AK13" s="17"/>
-      <c r="AL13" s="18"/>
-      <c r="AM13" s="18"/>
-      <c r="AN13" s="19"/>
-      <c r="AO13" s="17"/>
-      <c r="AP13" s="18"/>
-      <c r="AQ13" s="18"/>
-      <c r="AR13" s="19"/>
-      <c r="AS13" s="17"/>
-      <c r="AT13" s="18"/>
-      <c r="AU13" s="18"/>
-      <c r="AV13" s="19"/>
-      <c r="AW13" s="17"/>
-      <c r="AX13" s="18"/>
-      <c r="AY13" s="18"/>
-      <c r="AZ13" s="19"/>
-    </row>
-    <row r="14" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="68" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="47"/>
-      <c r="D14" s="48"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="8"/>
-      <c r="N14" s="21"/>
-      <c r="O14" s="29"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="21"/>
-      <c r="S14" s="29"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="8"/>
-      <c r="V14" s="21"/>
-      <c r="W14" s="29"/>
-      <c r="X14" s="10"/>
-      <c r="Y14" s="8"/>
-      <c r="Z14" s="21"/>
-      <c r="AA14" s="29"/>
-      <c r="AB14" s="10"/>
-      <c r="AC14" s="8"/>
-      <c r="AD14" s="21"/>
-      <c r="AE14" s="29"/>
-      <c r="AF14" s="10"/>
-      <c r="AG14" s="8"/>
-      <c r="AH14" s="21"/>
-      <c r="AI14" s="29"/>
-      <c r="AJ14" s="10"/>
-      <c r="AK14" s="8"/>
-      <c r="AL14" s="21"/>
-      <c r="AM14" s="29"/>
-      <c r="AN14" s="10"/>
-      <c r="AO14" s="8"/>
-      <c r="AP14" s="21"/>
-      <c r="AQ14" s="29"/>
-      <c r="AR14" s="10"/>
-      <c r="AS14" s="8"/>
-      <c r="AT14" s="21"/>
-      <c r="AU14" s="29"/>
-      <c r="AV14" s="10"/>
-      <c r="AW14" s="8"/>
-      <c r="AX14" s="21"/>
-      <c r="AY14" s="29"/>
-      <c r="AZ14" s="10"/>
-    </row>
-    <row r="15" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="43"/>
-      <c r="B15" s="53"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+    <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="62"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="42"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="13"/>
+      <c r="U13" s="11"/>
+      <c r="V13" s="12"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="13"/>
+      <c r="Y13" s="11"/>
+      <c r="Z13" s="12"/>
+      <c r="AA13" s="12"/>
+      <c r="AB13" s="13"/>
+      <c r="AC13" s="11"/>
+      <c r="AD13" s="12"/>
+      <c r="AE13" s="12"/>
+      <c r="AF13" s="13"/>
+      <c r="AG13" s="11"/>
+      <c r="AH13" s="12"/>
+      <c r="AI13" s="12"/>
+      <c r="AJ13" s="13"/>
+      <c r="AK13" s="11"/>
+      <c r="AL13" s="12"/>
+      <c r="AM13" s="12"/>
+      <c r="AN13" s="13"/>
+      <c r="AO13" s="11"/>
+      <c r="AP13" s="12"/>
+      <c r="AQ13" s="12"/>
+      <c r="AR13" s="13"/>
+      <c r="AS13" s="11"/>
+      <c r="AT13" s="12"/>
+      <c r="AU13" s="12"/>
+      <c r="AV13" s="13"/>
+      <c r="AW13" s="11"/>
+      <c r="AX13" s="12"/>
+      <c r="AY13" s="12"/>
+      <c r="AZ13" s="13"/>
+    </row>
+    <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="62"/>
+      <c r="B14" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="13"/>
+      <c r="U14" s="11"/>
+      <c r="V14" s="12"/>
+      <c r="W14" s="12"/>
+      <c r="X14" s="13"/>
+      <c r="Y14" s="11"/>
+      <c r="Z14" s="12"/>
+      <c r="AA14" s="12"/>
+      <c r="AB14" s="13"/>
+      <c r="AC14" s="11"/>
+      <c r="AD14" s="12"/>
+      <c r="AE14" s="12"/>
+      <c r="AF14" s="13"/>
+      <c r="AG14" s="11"/>
+      <c r="AH14" s="12"/>
+      <c r="AI14" s="12"/>
+      <c r="AJ14" s="13"/>
+      <c r="AK14" s="11"/>
+      <c r="AL14" s="12"/>
+      <c r="AM14" s="12"/>
+      <c r="AN14" s="13"/>
+      <c r="AO14" s="11"/>
+      <c r="AP14" s="12"/>
+      <c r="AQ14" s="12"/>
+      <c r="AR14" s="13"/>
+      <c r="AS14" s="11"/>
+      <c r="AT14" s="12"/>
+      <c r="AU14" s="12"/>
+      <c r="AV14" s="13"/>
+      <c r="AW14" s="11"/>
+      <c r="AX14" s="12"/>
+      <c r="AY14" s="12"/>
+      <c r="AZ14" s="13"/>
+    </row>
+    <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="62"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
       <c r="H15" s="13"/>
       <c r="I15" s="11"/>
       <c r="J15" s="12"/>
@@ -2236,164 +2242,177 @@
       <c r="AY15" s="12"/>
       <c r="AZ15" s="13"/>
     </row>
-    <row r="16" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A16" s="43"/>
-      <c r="B16" s="46" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" s="41"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="11"/>
+    <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="62"/>
+      <c r="B16" s="86"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="51"/>
+      <c r="E16" s="20"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
-      <c r="I16" s="11"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="20"/>
       <c r="J16" s="12"/>
       <c r="K16" s="12"/>
-      <c r="M16" s="11"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="20"/>
       <c r="N16" s="12"/>
       <c r="O16" s="12"/>
-      <c r="Q16" s="11"/>
+      <c r="P16" s="13"/>
+      <c r="Q16" s="20"/>
       <c r="R16" s="12"/>
       <c r="S16" s="12"/>
-      <c r="U16" s="11"/>
+      <c r="T16" s="13"/>
+      <c r="U16" s="20"/>
       <c r="V16" s="12"/>
       <c r="W16" s="12"/>
-      <c r="Y16" s="11"/>
+      <c r="X16" s="13"/>
+      <c r="Y16" s="20"/>
       <c r="Z16" s="12"/>
       <c r="AA16" s="12"/>
-      <c r="AC16" s="11"/>
+      <c r="AB16" s="13"/>
+      <c r="AC16" s="20"/>
       <c r="AD16" s="12"/>
       <c r="AE16" s="12"/>
-      <c r="AG16" s="11"/>
+      <c r="AF16" s="13"/>
+      <c r="AG16" s="20"/>
       <c r="AH16" s="12"/>
       <c r="AI16" s="12"/>
-      <c r="AK16" s="11"/>
+      <c r="AJ16" s="13"/>
+      <c r="AK16" s="20"/>
       <c r="AL16" s="12"/>
       <c r="AM16" s="12"/>
-      <c r="AO16" s="11"/>
+      <c r="AN16" s="13"/>
+      <c r="AO16" s="20"/>
       <c r="AP16" s="12"/>
       <c r="AQ16" s="12"/>
-      <c r="AS16" s="11"/>
+      <c r="AR16" s="13"/>
+      <c r="AS16" s="20"/>
       <c r="AT16" s="12"/>
       <c r="AU16" s="12"/>
-      <c r="AW16" s="11"/>
+      <c r="AV16" s="13"/>
+      <c r="AW16" s="20"/>
       <c r="AX16" s="12"/>
       <c r="AY16" s="12"/>
       <c r="AZ16" s="13"/>
     </row>
-    <row r="17" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A17" s="43"/>
-      <c r="B17" s="46"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="12"/>
-      <c r="O17" s="12"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="12"/>
-      <c r="S17" s="12"/>
-      <c r="T17" s="13"/>
-      <c r="U17" s="11"/>
-      <c r="V17" s="12"/>
-      <c r="W17" s="12"/>
-      <c r="X17" s="13"/>
-      <c r="Y17" s="11"/>
-      <c r="Z17" s="12"/>
-      <c r="AA17" s="12"/>
-      <c r="AB17" s="13"/>
-      <c r="AC17" s="11"/>
-      <c r="AD17" s="12"/>
-      <c r="AE17" s="12"/>
-      <c r="AF17" s="13"/>
-      <c r="AG17" s="11"/>
-      <c r="AH17" s="12"/>
-      <c r="AI17" s="12"/>
-      <c r="AJ17" s="13"/>
-      <c r="AK17" s="11"/>
-      <c r="AL17" s="12"/>
-      <c r="AM17" s="12"/>
-      <c r="AN17" s="13"/>
-      <c r="AO17" s="11"/>
-      <c r="AP17" s="12"/>
-      <c r="AQ17" s="12"/>
-      <c r="AR17" s="13"/>
-      <c r="AS17" s="11"/>
-      <c r="AT17" s="12"/>
-      <c r="AU17" s="12"/>
-      <c r="AV17" s="13"/>
-      <c r="AW17" s="11"/>
-      <c r="AX17" s="12"/>
-      <c r="AY17" s="12"/>
-      <c r="AZ17" s="13"/>
-    </row>
-    <row r="18" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A18" s="43"/>
-      <c r="B18" s="46"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="11"/>
-      <c r="R18" s="12"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="11"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="12"/>
-      <c r="X18" s="13"/>
-      <c r="Y18" s="11"/>
-      <c r="Z18" s="12"/>
-      <c r="AA18" s="12"/>
-      <c r="AB18" s="13"/>
-      <c r="AC18" s="11"/>
-      <c r="AD18" s="12"/>
-      <c r="AE18" s="12"/>
-      <c r="AF18" s="13"/>
-      <c r="AG18" s="11"/>
-      <c r="AH18" s="12"/>
-      <c r="AI18" s="12"/>
-      <c r="AJ18" s="13"/>
-      <c r="AK18" s="11"/>
-      <c r="AL18" s="12"/>
-      <c r="AM18" s="12"/>
-      <c r="AN18" s="13"/>
-      <c r="AO18" s="11"/>
-      <c r="AP18" s="12"/>
-      <c r="AQ18" s="12"/>
-      <c r="AR18" s="13"/>
-      <c r="AS18" s="11"/>
-      <c r="AT18" s="12"/>
-      <c r="AU18" s="12"/>
-      <c r="AV18" s="13"/>
-      <c r="AW18" s="11"/>
-      <c r="AX18" s="12"/>
-      <c r="AY18" s="12"/>
-      <c r="AZ18" s="13"/>
-    </row>
-    <row r="19" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A19" s="43"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="49"/>
+    <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="63"/>
+      <c r="B17" s="93"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="18"/>
+      <c r="S17" s="18"/>
+      <c r="T17" s="19"/>
+      <c r="U17" s="17"/>
+      <c r="V17" s="18"/>
+      <c r="W17" s="18"/>
+      <c r="X17" s="19"/>
+      <c r="Y17" s="17"/>
+      <c r="Z17" s="18"/>
+      <c r="AA17" s="18"/>
+      <c r="AB17" s="19"/>
+      <c r="AC17" s="17"/>
+      <c r="AD17" s="18"/>
+      <c r="AE17" s="18"/>
+      <c r="AF17" s="19"/>
+      <c r="AG17" s="17"/>
+      <c r="AH17" s="18"/>
+      <c r="AI17" s="18"/>
+      <c r="AJ17" s="19"/>
+      <c r="AK17" s="17"/>
+      <c r="AL17" s="18"/>
+      <c r="AM17" s="18"/>
+      <c r="AN17" s="19"/>
+      <c r="AO17" s="17"/>
+      <c r="AP17" s="18"/>
+      <c r="AQ17" s="18"/>
+      <c r="AR17" s="19"/>
+      <c r="AS17" s="17"/>
+      <c r="AT17" s="18"/>
+      <c r="AU17" s="18"/>
+      <c r="AV17" s="19"/>
+      <c r="AW17" s="17"/>
+      <c r="AX17" s="18"/>
+      <c r="AY17" s="18"/>
+      <c r="AZ17" s="19"/>
+    </row>
+    <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="61" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="83" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="81"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="29"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="29"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="29"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="29"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="8"/>
+      <c r="V18" s="21"/>
+      <c r="W18" s="29"/>
+      <c r="X18" s="10"/>
+      <c r="Y18" s="8"/>
+      <c r="Z18" s="21"/>
+      <c r="AA18" s="29"/>
+      <c r="AB18" s="10"/>
+      <c r="AC18" s="8"/>
+      <c r="AD18" s="21"/>
+      <c r="AE18" s="29"/>
+      <c r="AF18" s="10"/>
+      <c r="AG18" s="8"/>
+      <c r="AH18" s="21"/>
+      <c r="AI18" s="29"/>
+      <c r="AJ18" s="10"/>
+      <c r="AK18" s="8"/>
+      <c r="AL18" s="21"/>
+      <c r="AM18" s="29"/>
+      <c r="AN18" s="10"/>
+      <c r="AO18" s="8"/>
+      <c r="AP18" s="21"/>
+      <c r="AQ18" s="29"/>
+      <c r="AR18" s="10"/>
+      <c r="AS18" s="8"/>
+      <c r="AT18" s="21"/>
+      <c r="AU18" s="29"/>
+      <c r="AV18" s="10"/>
+      <c r="AW18" s="8"/>
+      <c r="AX18" s="21"/>
+      <c r="AY18" s="29"/>
+      <c r="AZ18" s="10"/>
+    </row>
+    <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="62"/>
+      <c r="B19" s="84"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="51"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2443,615 +2462,606 @@
       <c r="AY19" s="12"/>
       <c r="AZ19" s="13"/>
     </row>
-    <row r="20" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="43"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="56"/>
-      <c r="D20" s="60"/>
+    <row r="20" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A20" s="62"/>
+      <c r="B20" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="54"/>
+      <c r="D20" s="51"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
-      <c r="H20" s="13"/>
       <c r="I20" s="11"/>
       <c r="J20" s="12"/>
       <c r="K20" s="12"/>
-      <c r="L20" s="13"/>
       <c r="M20" s="11"/>
       <c r="N20" s="12"/>
       <c r="O20" s="12"/>
-      <c r="P20" s="13"/>
       <c r="Q20" s="11"/>
       <c r="R20" s="12"/>
       <c r="S20" s="12"/>
-      <c r="T20" s="13"/>
       <c r="U20" s="11"/>
       <c r="V20" s="12"/>
       <c r="W20" s="12"/>
-      <c r="X20" s="13"/>
       <c r="Y20" s="11"/>
       <c r="Z20" s="12"/>
       <c r="AA20" s="12"/>
-      <c r="AB20" s="13"/>
       <c r="AC20" s="11"/>
       <c r="AD20" s="12"/>
       <c r="AE20" s="12"/>
-      <c r="AF20" s="13"/>
       <c r="AG20" s="11"/>
       <c r="AH20" s="12"/>
       <c r="AI20" s="12"/>
-      <c r="AJ20" s="13"/>
       <c r="AK20" s="11"/>
       <c r="AL20" s="12"/>
       <c r="AM20" s="12"/>
-      <c r="AN20" s="13"/>
       <c r="AO20" s="11"/>
       <c r="AP20" s="12"/>
       <c r="AQ20" s="12"/>
-      <c r="AR20" s="13"/>
       <c r="AS20" s="11"/>
       <c r="AT20" s="12"/>
       <c r="AU20" s="12"/>
-      <c r="AV20" s="13"/>
       <c r="AW20" s="11"/>
       <c r="AX20" s="12"/>
       <c r="AY20" s="12"/>
       <c r="AZ20" s="13"/>
     </row>
-    <row r="21" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="43"/>
-      <c r="B21" s="46"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="61"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="15"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="16"/>
-      <c r="Q21" s="14"/>
-      <c r="R21" s="15"/>
-      <c r="S21" s="15"/>
-      <c r="T21" s="16"/>
-      <c r="U21" s="14"/>
-      <c r="V21" s="15"/>
-      <c r="W21" s="15"/>
-      <c r="X21" s="16"/>
-      <c r="Y21" s="14"/>
-      <c r="Z21" s="15"/>
-      <c r="AA21" s="15"/>
-      <c r="AB21" s="16"/>
-      <c r="AC21" s="14"/>
-      <c r="AD21" s="15"/>
-      <c r="AE21" s="15"/>
-      <c r="AF21" s="16"/>
-      <c r="AG21" s="14"/>
-      <c r="AH21" s="15"/>
-      <c r="AI21" s="15"/>
-      <c r="AJ21" s="16"/>
-      <c r="AK21" s="14"/>
-      <c r="AL21" s="15"/>
-      <c r="AM21" s="15"/>
-      <c r="AN21" s="16"/>
-      <c r="AO21" s="14"/>
-      <c r="AP21" s="15"/>
-      <c r="AQ21" s="15"/>
-      <c r="AR21" s="16"/>
-      <c r="AS21" s="14"/>
-      <c r="AT21" s="15"/>
-      <c r="AU21" s="15"/>
-      <c r="AV21" s="16"/>
-      <c r="AW21" s="14"/>
-      <c r="AX21" s="15"/>
-      <c r="AY21" s="15"/>
-      <c r="AZ21" s="16"/>
-    </row>
-    <row r="22" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="43"/>
-      <c r="B22" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="56"/>
-      <c r="D22" s="60">
+    <row r="21" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A21" s="62"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="11"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="11"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="13"/>
+      <c r="Y21" s="11"/>
+      <c r="Z21" s="12"/>
+      <c r="AA21" s="12"/>
+      <c r="AB21" s="13"/>
+      <c r="AC21" s="11"/>
+      <c r="AD21" s="12"/>
+      <c r="AE21" s="12"/>
+      <c r="AF21" s="13"/>
+      <c r="AG21" s="11"/>
+      <c r="AH21" s="12"/>
+      <c r="AI21" s="12"/>
+      <c r="AJ21" s="13"/>
+      <c r="AK21" s="11"/>
+      <c r="AL21" s="12"/>
+      <c r="AM21" s="12"/>
+      <c r="AN21" s="13"/>
+      <c r="AO21" s="11"/>
+      <c r="AP21" s="12"/>
+      <c r="AQ21" s="12"/>
+      <c r="AR21" s="13"/>
+      <c r="AS21" s="11"/>
+      <c r="AT21" s="12"/>
+      <c r="AU21" s="12"/>
+      <c r="AV21" s="13"/>
+      <c r="AW21" s="11"/>
+      <c r="AX21" s="12"/>
+      <c r="AY21" s="12"/>
+      <c r="AZ21" s="13"/>
+    </row>
+    <row r="22" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A22" s="62"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="12"/>
+      <c r="T22" s="13"/>
+      <c r="U22" s="11"/>
+      <c r="V22" s="12"/>
+      <c r="W22" s="12"/>
+      <c r="X22" s="13"/>
+      <c r="Y22" s="11"/>
+      <c r="Z22" s="12"/>
+      <c r="AA22" s="12"/>
+      <c r="AB22" s="13"/>
+      <c r="AC22" s="11"/>
+      <c r="AD22" s="12"/>
+      <c r="AE22" s="12"/>
+      <c r="AF22" s="13"/>
+      <c r="AG22" s="11"/>
+      <c r="AH22" s="12"/>
+      <c r="AI22" s="12"/>
+      <c r="AJ22" s="13"/>
+      <c r="AK22" s="11"/>
+      <c r="AL22" s="12"/>
+      <c r="AM22" s="12"/>
+      <c r="AN22" s="13"/>
+      <c r="AO22" s="11"/>
+      <c r="AP22" s="12"/>
+      <c r="AQ22" s="12"/>
+      <c r="AR22" s="13"/>
+      <c r="AS22" s="11"/>
+      <c r="AT22" s="12"/>
+      <c r="AU22" s="12"/>
+      <c r="AV22" s="13"/>
+      <c r="AW22" s="11"/>
+      <c r="AX22" s="12"/>
+      <c r="AY22" s="12"/>
+      <c r="AZ22" s="13"/>
+    </row>
+    <row r="23" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A23" s="62"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="51"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="11"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="13"/>
+      <c r="U23" s="11"/>
+      <c r="V23" s="12"/>
+      <c r="W23" s="12"/>
+      <c r="X23" s="13"/>
+      <c r="Y23" s="11"/>
+      <c r="Z23" s="12"/>
+      <c r="AA23" s="12"/>
+      <c r="AB23" s="13"/>
+      <c r="AC23" s="11"/>
+      <c r="AD23" s="12"/>
+      <c r="AE23" s="12"/>
+      <c r="AF23" s="13"/>
+      <c r="AG23" s="11"/>
+      <c r="AH23" s="12"/>
+      <c r="AI23" s="12"/>
+      <c r="AJ23" s="13"/>
+      <c r="AK23" s="11"/>
+      <c r="AL23" s="12"/>
+      <c r="AM23" s="12"/>
+      <c r="AN23" s="13"/>
+      <c r="AO23" s="11"/>
+      <c r="AP23" s="12"/>
+      <c r="AQ23" s="12"/>
+      <c r="AR23" s="13"/>
+      <c r="AS23" s="11"/>
+      <c r="AT23" s="12"/>
+      <c r="AU23" s="12"/>
+      <c r="AV23" s="13"/>
+      <c r="AW23" s="11"/>
+      <c r="AX23" s="12"/>
+      <c r="AY23" s="12"/>
+      <c r="AZ23" s="13"/>
+    </row>
+    <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="62"/>
+      <c r="B24" s="86"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="11"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="13"/>
+      <c r="U24" s="11"/>
+      <c r="V24" s="12"/>
+      <c r="W24" s="12"/>
+      <c r="X24" s="13"/>
+      <c r="Y24" s="11"/>
+      <c r="Z24" s="12"/>
+      <c r="AA24" s="12"/>
+      <c r="AB24" s="13"/>
+      <c r="AC24" s="11"/>
+      <c r="AD24" s="12"/>
+      <c r="AE24" s="12"/>
+      <c r="AF24" s="13"/>
+      <c r="AG24" s="11"/>
+      <c r="AH24" s="12"/>
+      <c r="AI24" s="12"/>
+      <c r="AJ24" s="13"/>
+      <c r="AK24" s="11"/>
+      <c r="AL24" s="12"/>
+      <c r="AM24" s="12"/>
+      <c r="AN24" s="13"/>
+      <c r="AO24" s="11"/>
+      <c r="AP24" s="12"/>
+      <c r="AQ24" s="12"/>
+      <c r="AR24" s="13"/>
+      <c r="AS24" s="11"/>
+      <c r="AT24" s="12"/>
+      <c r="AU24" s="12"/>
+      <c r="AV24" s="13"/>
+      <c r="AW24" s="11"/>
+      <c r="AX24" s="12"/>
+      <c r="AY24" s="12"/>
+      <c r="AZ24" s="13"/>
+    </row>
+    <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="62"/>
+      <c r="B25" s="72"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="89"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="14"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="15"/>
+      <c r="P25" s="16"/>
+      <c r="Q25" s="14"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+      <c r="T25" s="16"/>
+      <c r="U25" s="14"/>
+      <c r="V25" s="15"/>
+      <c r="W25" s="15"/>
+      <c r="X25" s="16"/>
+      <c r="Y25" s="14"/>
+      <c r="Z25" s="15"/>
+      <c r="AA25" s="15"/>
+      <c r="AB25" s="16"/>
+      <c r="AC25" s="14"/>
+      <c r="AD25" s="15"/>
+      <c r="AE25" s="15"/>
+      <c r="AF25" s="16"/>
+      <c r="AG25" s="14"/>
+      <c r="AH25" s="15"/>
+      <c r="AI25" s="15"/>
+      <c r="AJ25" s="16"/>
+      <c r="AK25" s="14"/>
+      <c r="AL25" s="15"/>
+      <c r="AM25" s="15"/>
+      <c r="AN25" s="16"/>
+      <c r="AO25" s="14"/>
+      <c r="AP25" s="15"/>
+      <c r="AQ25" s="15"/>
+      <c r="AR25" s="16"/>
+      <c r="AS25" s="14"/>
+      <c r="AT25" s="15"/>
+      <c r="AU25" s="15"/>
+      <c r="AV25" s="16"/>
+      <c r="AW25" s="14"/>
+      <c r="AX25" s="15"/>
+      <c r="AY25" s="15"/>
+      <c r="AZ25" s="16"/>
+    </row>
+    <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="62"/>
+      <c r="B26" s="52" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="64"/>
+      <c r="D26" s="88">
         <v>0</v>
       </c>
-      <c r="E22" s="14"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="16"/>
-      <c r="Q22" s="14"/>
-      <c r="R22" s="15"/>
-      <c r="S22" s="15"/>
-      <c r="T22" s="16"/>
-      <c r="U22" s="14"/>
-      <c r="V22" s="15"/>
-      <c r="W22" s="15"/>
-      <c r="X22" s="16"/>
-      <c r="Y22" s="14"/>
-      <c r="Z22" s="15"/>
-      <c r="AA22" s="15"/>
-      <c r="AB22" s="16"/>
-      <c r="AC22" s="14"/>
-      <c r="AD22" s="15"/>
-      <c r="AE22" s="15"/>
-      <c r="AF22" s="16"/>
-      <c r="AG22" s="14"/>
-      <c r="AH22" s="15"/>
-      <c r="AI22" s="15"/>
-      <c r="AJ22" s="16"/>
-      <c r="AK22" s="14"/>
-      <c r="AL22" s="15"/>
-      <c r="AM22" s="15"/>
-      <c r="AN22" s="16"/>
-      <c r="AO22" s="14"/>
-      <c r="AP22" s="15"/>
-      <c r="AQ22" s="15"/>
-      <c r="AR22" s="16"/>
-      <c r="AS22" s="14"/>
-      <c r="AT22" s="15"/>
-      <c r="AU22" s="15"/>
-      <c r="AV22" s="16"/>
-      <c r="AW22" s="14"/>
-      <c r="AX22" s="15"/>
-      <c r="AY22" s="15"/>
-      <c r="AZ22" s="16"/>
-    </row>
-    <row r="23" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="44"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="79"/>
-      <c r="D23" s="62"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="17"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="18"/>
-      <c r="T23" s="19"/>
-      <c r="U23" s="17"/>
-      <c r="V23" s="18"/>
-      <c r="W23" s="18"/>
-      <c r="X23" s="19"/>
-      <c r="Y23" s="17"/>
-      <c r="Z23" s="18"/>
-      <c r="AA23" s="18"/>
-      <c r="AB23" s="19"/>
-      <c r="AC23" s="17"/>
-      <c r="AD23" s="18"/>
-      <c r="AE23" s="18"/>
-      <c r="AF23" s="19"/>
-      <c r="AG23" s="17"/>
-      <c r="AH23" s="18"/>
-      <c r="AI23" s="18"/>
-      <c r="AJ23" s="19"/>
-      <c r="AK23" s="17"/>
-      <c r="AL23" s="18"/>
-      <c r="AM23" s="18"/>
-      <c r="AN23" s="19"/>
-      <c r="AO23" s="17"/>
-      <c r="AP23" s="18"/>
-      <c r="AQ23" s="18"/>
-      <c r="AR23" s="19"/>
-      <c r="AS23" s="17"/>
-      <c r="AT23" s="18"/>
-      <c r="AU23" s="18"/>
-      <c r="AV23" s="19"/>
-      <c r="AW23" s="17"/>
-      <c r="AX23" s="18"/>
-      <c r="AY23" s="18"/>
-      <c r="AZ23" s="19"/>
-    </row>
-    <row r="24" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A24" s="42" t="s">
+      <c r="E26" s="14"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="15"/>
+      <c r="K26" s="15"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="14"/>
+      <c r="N26" s="15"/>
+      <c r="O26" s="15"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="14"/>
+      <c r="R26" s="15"/>
+      <c r="S26" s="15"/>
+      <c r="T26" s="16"/>
+      <c r="U26" s="14"/>
+      <c r="V26" s="15"/>
+      <c r="W26" s="15"/>
+      <c r="X26" s="16"/>
+      <c r="Y26" s="14"/>
+      <c r="Z26" s="15"/>
+      <c r="AA26" s="15"/>
+      <c r="AB26" s="16"/>
+      <c r="AC26" s="14"/>
+      <c r="AD26" s="15"/>
+      <c r="AE26" s="15"/>
+      <c r="AF26" s="16"/>
+      <c r="AG26" s="14"/>
+      <c r="AH26" s="15"/>
+      <c r="AI26" s="15"/>
+      <c r="AJ26" s="16"/>
+      <c r="AK26" s="14"/>
+      <c r="AL26" s="15"/>
+      <c r="AM26" s="15"/>
+      <c r="AN26" s="16"/>
+      <c r="AO26" s="14"/>
+      <c r="AP26" s="15"/>
+      <c r="AQ26" s="15"/>
+      <c r="AR26" s="16"/>
+      <c r="AS26" s="14"/>
+      <c r="AT26" s="15"/>
+      <c r="AU26" s="15"/>
+      <c r="AV26" s="16"/>
+      <c r="AW26" s="14"/>
+      <c r="AX26" s="15"/>
+      <c r="AY26" s="15"/>
+      <c r="AZ26" s="16"/>
+    </row>
+    <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="63"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="77"/>
+      <c r="D27" s="90"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="17"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="18"/>
+      <c r="P27" s="19"/>
+      <c r="Q27" s="17"/>
+      <c r="R27" s="18"/>
+      <c r="S27" s="18"/>
+      <c r="T27" s="19"/>
+      <c r="U27" s="17"/>
+      <c r="V27" s="18"/>
+      <c r="W27" s="18"/>
+      <c r="X27" s="19"/>
+      <c r="Y27" s="17"/>
+      <c r="Z27" s="18"/>
+      <c r="AA27" s="18"/>
+      <c r="AB27" s="19"/>
+      <c r="AC27" s="17"/>
+      <c r="AD27" s="18"/>
+      <c r="AE27" s="18"/>
+      <c r="AF27" s="19"/>
+      <c r="AG27" s="17"/>
+      <c r="AH27" s="18"/>
+      <c r="AI27" s="18"/>
+      <c r="AJ27" s="19"/>
+      <c r="AK27" s="17"/>
+      <c r="AL27" s="18"/>
+      <c r="AM27" s="18"/>
+      <c r="AN27" s="19"/>
+      <c r="AO27" s="17"/>
+      <c r="AP27" s="18"/>
+      <c r="AQ27" s="18"/>
+      <c r="AR27" s="19"/>
+      <c r="AS27" s="17"/>
+      <c r="AT27" s="18"/>
+      <c r="AU27" s="18"/>
+      <c r="AV27" s="19"/>
+      <c r="AW27" s="17"/>
+      <c r="AX27" s="18"/>
+      <c r="AY27" s="18"/>
+      <c r="AZ27" s="19"/>
+    </row>
+    <row r="28" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A28" s="61" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="80" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="81"/>
+      <c r="D28" s="82"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="9"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="9"/>
+      <c r="S28" s="9"/>
+      <c r="T28" s="10"/>
+      <c r="U28" s="8"/>
+      <c r="V28" s="9"/>
+      <c r="W28" s="9"/>
+      <c r="X28" s="10"/>
+      <c r="Y28" s="8"/>
+      <c r="Z28" s="9"/>
+      <c r="AA28" s="9"/>
+      <c r="AB28" s="10"/>
+      <c r="AC28" s="8"/>
+      <c r="AD28" s="9"/>
+      <c r="AE28" s="9"/>
+      <c r="AF28" s="10"/>
+      <c r="AG28" s="8"/>
+      <c r="AH28" s="9"/>
+      <c r="AI28" s="9"/>
+      <c r="AJ28" s="10"/>
+      <c r="AK28" s="8"/>
+      <c r="AL28" s="9"/>
+      <c r="AM28" s="9"/>
+      <c r="AN28" s="10"/>
+      <c r="AO28" s="8"/>
+      <c r="AP28" s="9"/>
+      <c r="AQ28" s="9"/>
+      <c r="AR28" s="10"/>
+      <c r="AS28" s="8"/>
+      <c r="AT28" s="9"/>
+      <c r="AU28" s="9"/>
+      <c r="AV28" s="10"/>
+      <c r="AW28" s="8"/>
+      <c r="AX28" s="9"/>
+      <c r="AY28" s="9"/>
+      <c r="AZ28" s="10"/>
+    </row>
+    <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="62"/>
+      <c r="B29" s="73"/>
+      <c r="C29" s="74"/>
+      <c r="D29" s="75"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="18"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="17"/>
+      <c r="R29" s="18"/>
+      <c r="S29" s="18"/>
+      <c r="T29" s="19"/>
+      <c r="U29" s="17"/>
+      <c r="V29" s="18"/>
+      <c r="W29" s="18"/>
+      <c r="X29" s="19"/>
+      <c r="Y29" s="17"/>
+      <c r="Z29" s="18"/>
+      <c r="AA29" s="18"/>
+      <c r="AB29" s="19"/>
+      <c r="AC29" s="17"/>
+      <c r="AD29" s="18"/>
+      <c r="AE29" s="18"/>
+      <c r="AF29" s="19"/>
+      <c r="AG29" s="17"/>
+      <c r="AH29" s="18"/>
+      <c r="AI29" s="18"/>
+      <c r="AJ29" s="19"/>
+      <c r="AK29" s="17"/>
+      <c r="AL29" s="18"/>
+      <c r="AM29" s="18"/>
+      <c r="AN29" s="19"/>
+      <c r="AO29" s="17"/>
+      <c r="AP29" s="18"/>
+      <c r="AQ29" s="18"/>
+      <c r="AR29" s="19"/>
+      <c r="AS29" s="17"/>
+      <c r="AT29" s="18"/>
+      <c r="AU29" s="18"/>
+      <c r="AV29" s="19"/>
+      <c r="AW29" s="17"/>
+      <c r="AX29" s="18"/>
+      <c r="AY29" s="18"/>
+      <c r="AZ29" s="19"/>
+    </row>
+    <row r="30" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A30" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="C24" s="47"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="8"/>
-      <c r="R24" s="9"/>
-      <c r="S24" s="9"/>
-      <c r="T24" s="10"/>
-      <c r="U24" s="8"/>
-      <c r="V24" s="9"/>
-      <c r="W24" s="9"/>
-      <c r="X24" s="10"/>
-      <c r="Y24" s="8"/>
-      <c r="Z24" s="9"/>
-      <c r="AA24" s="9"/>
-      <c r="AB24" s="10"/>
-      <c r="AC24" s="8"/>
-      <c r="AD24" s="9"/>
-      <c r="AE24" s="9"/>
-      <c r="AF24" s="10"/>
-      <c r="AG24" s="8"/>
-      <c r="AH24" s="9"/>
-      <c r="AI24" s="9"/>
-      <c r="AJ24" s="10"/>
-      <c r="AK24" s="8"/>
-      <c r="AL24" s="9"/>
-      <c r="AM24" s="9"/>
-      <c r="AN24" s="10"/>
-      <c r="AO24" s="8"/>
-      <c r="AP24" s="9"/>
-      <c r="AQ24" s="9"/>
-      <c r="AR24" s="10"/>
-      <c r="AS24" s="8"/>
-      <c r="AT24" s="9"/>
-      <c r="AU24" s="9"/>
-      <c r="AV24" s="10"/>
-      <c r="AW24" s="8"/>
-      <c r="AX24" s="9"/>
-      <c r="AY24" s="9"/>
-      <c r="AZ24" s="10"/>
-    </row>
-    <row r="25" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="43"/>
-      <c r="B25" s="50"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="17"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="18"/>
-      <c r="O25" s="18"/>
-      <c r="P25" s="19"/>
-      <c r="Q25" s="17"/>
-      <c r="R25" s="18"/>
-      <c r="S25" s="18"/>
-      <c r="T25" s="19"/>
-      <c r="U25" s="17"/>
-      <c r="V25" s="18"/>
-      <c r="W25" s="18"/>
-      <c r="X25" s="19"/>
-      <c r="Y25" s="17"/>
-      <c r="Z25" s="18"/>
-      <c r="AA25" s="18"/>
-      <c r="AB25" s="19"/>
-      <c r="AC25" s="17"/>
-      <c r="AD25" s="18"/>
-      <c r="AE25" s="18"/>
-      <c r="AF25" s="19"/>
-      <c r="AG25" s="17"/>
-      <c r="AH25" s="18"/>
-      <c r="AI25" s="18"/>
-      <c r="AJ25" s="19"/>
-      <c r="AK25" s="17"/>
-      <c r="AL25" s="18"/>
-      <c r="AM25" s="18"/>
-      <c r="AN25" s="19"/>
-      <c r="AO25" s="17"/>
-      <c r="AP25" s="18"/>
-      <c r="AQ25" s="18"/>
-      <c r="AR25" s="19"/>
-      <c r="AS25" s="17"/>
-      <c r="AT25" s="18"/>
-      <c r="AU25" s="18"/>
-      <c r="AV25" s="19"/>
-      <c r="AW25" s="17"/>
-      <c r="AX25" s="18"/>
-      <c r="AY25" s="18"/>
-      <c r="AZ25" s="19"/>
-    </row>
-    <row r="26" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A26" s="42" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="8"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="10"/>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="9"/>
-      <c r="S26" s="9"/>
-      <c r="T26" s="10"/>
-      <c r="U26" s="8"/>
-      <c r="V26" s="9"/>
-      <c r="W26" s="9"/>
-      <c r="X26" s="10"/>
-      <c r="Y26" s="8"/>
-      <c r="Z26" s="9"/>
-      <c r="AA26" s="9"/>
-      <c r="AB26" s="10"/>
-      <c r="AC26" s="8"/>
-      <c r="AD26" s="9"/>
-      <c r="AE26" s="9"/>
-      <c r="AF26" s="10"/>
-      <c r="AG26" s="8"/>
-      <c r="AH26" s="9"/>
-      <c r="AI26" s="9"/>
-      <c r="AJ26" s="10"/>
-      <c r="AK26" s="8"/>
-      <c r="AL26" s="9"/>
-      <c r="AM26" s="9"/>
-      <c r="AN26" s="10"/>
-      <c r="AO26" s="8"/>
-      <c r="AP26" s="9"/>
-      <c r="AQ26" s="9"/>
-      <c r="AR26" s="10"/>
-      <c r="AS26" s="8"/>
-      <c r="AT26" s="9"/>
-      <c r="AU26" s="9"/>
-      <c r="AV26" s="10"/>
-      <c r="AW26" s="8"/>
-      <c r="AX26" s="9"/>
-      <c r="AY26" s="9"/>
-      <c r="AZ26" s="10"/>
-    </row>
-    <row r="27" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A27" s="43"/>
-      <c r="B27" s="46"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="12"/>
-      <c r="O27" s="12"/>
-      <c r="P27" s="13"/>
-      <c r="Q27" s="11"/>
-      <c r="R27" s="12"/>
-      <c r="S27" s="12"/>
-      <c r="T27" s="13"/>
-      <c r="U27" s="11"/>
-      <c r="V27" s="12"/>
-      <c r="W27" s="12"/>
-      <c r="X27" s="13"/>
-      <c r="Y27" s="11"/>
-      <c r="Z27" s="12"/>
-      <c r="AA27" s="12"/>
-      <c r="AB27" s="13"/>
-      <c r="AC27" s="11"/>
-      <c r="AD27" s="12"/>
-      <c r="AE27" s="12"/>
-      <c r="AF27" s="13"/>
-      <c r="AG27" s="11"/>
-      <c r="AH27" s="12"/>
-      <c r="AI27" s="12"/>
-      <c r="AJ27" s="13"/>
-      <c r="AK27" s="11"/>
-      <c r="AL27" s="12"/>
-      <c r="AM27" s="12"/>
-      <c r="AN27" s="13"/>
-      <c r="AO27" s="11"/>
-      <c r="AP27" s="12"/>
-      <c r="AQ27" s="12"/>
-      <c r="AR27" s="13"/>
-      <c r="AS27" s="11"/>
-      <c r="AT27" s="12"/>
-      <c r="AU27" s="12"/>
-      <c r="AV27" s="13"/>
-      <c r="AW27" s="11"/>
-      <c r="AX27" s="12"/>
-      <c r="AY27" s="12"/>
-      <c r="AZ27" s="13"/>
-    </row>
-    <row r="28" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="43"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="41"/>
-      <c r="D28" s="49"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="L28" s="13"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="12"/>
-      <c r="O28" s="12"/>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="11"/>
-      <c r="R28" s="12"/>
-      <c r="S28" s="12"/>
-      <c r="T28" s="13"/>
-      <c r="U28" s="11"/>
-      <c r="V28" s="12"/>
-      <c r="W28" s="12"/>
-      <c r="X28" s="13"/>
-      <c r="Y28" s="11"/>
-      <c r="Z28" s="12"/>
-      <c r="AA28" s="12"/>
-      <c r="AB28" s="13"/>
-      <c r="AC28" s="11"/>
-      <c r="AD28" s="12"/>
-      <c r="AE28" s="12"/>
-      <c r="AF28" s="13"/>
-      <c r="AG28" s="11"/>
-      <c r="AH28" s="12"/>
-      <c r="AI28" s="12"/>
-      <c r="AJ28" s="13"/>
-      <c r="AK28" s="11"/>
-      <c r="AL28" s="12"/>
-      <c r="AM28" s="12"/>
-      <c r="AN28" s="13"/>
-      <c r="AO28" s="11"/>
-      <c r="AP28" s="12"/>
-      <c r="AQ28" s="12"/>
-      <c r="AR28" s="13"/>
-      <c r="AS28" s="11"/>
-      <c r="AT28" s="12"/>
-      <c r="AU28" s="12"/>
-      <c r="AV28" s="13"/>
-      <c r="AW28" s="11"/>
-      <c r="AX28" s="12"/>
-      <c r="AY28" s="12"/>
-      <c r="AZ28" s="13"/>
-    </row>
-    <row r="29" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="43"/>
-      <c r="B29" s="39"/>
-      <c r="C29" s="41"/>
-      <c r="D29" s="49"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="12"/>
-      <c r="O29" s="12"/>
-      <c r="P29" s="13"/>
-      <c r="Q29" s="11"/>
-      <c r="R29" s="12"/>
-      <c r="S29" s="12"/>
-      <c r="T29" s="13"/>
-      <c r="U29" s="11"/>
-      <c r="V29" s="12"/>
-      <c r="W29" s="12"/>
-      <c r="X29" s="13"/>
-      <c r="Y29" s="11"/>
-      <c r="Z29" s="12"/>
-      <c r="AA29" s="12"/>
-      <c r="AB29" s="13"/>
-      <c r="AC29" s="11"/>
-      <c r="AD29" s="12"/>
-      <c r="AE29" s="12"/>
-      <c r="AF29" s="13"/>
-      <c r="AG29" s="11"/>
-      <c r="AH29" s="12"/>
-      <c r="AI29" s="12"/>
-      <c r="AJ29" s="13"/>
-      <c r="AK29" s="11"/>
-      <c r="AL29" s="12"/>
-      <c r="AM29" s="12"/>
-      <c r="AN29" s="13"/>
-      <c r="AO29" s="11"/>
-      <c r="AP29" s="12"/>
-      <c r="AQ29" s="12"/>
-      <c r="AR29" s="13"/>
-      <c r="AS29" s="11"/>
-      <c r="AT29" s="12"/>
-      <c r="AU29" s="12"/>
-      <c r="AV29" s="13"/>
-      <c r="AW29" s="11"/>
-      <c r="AX29" s="12"/>
-      <c r="AY29" s="12"/>
-      <c r="AZ29" s="13"/>
-    </row>
-    <row r="30" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A30" s="43"/>
-      <c r="B30" s="38"/>
-      <c r="C30" s="40"/>
-      <c r="D30" s="49"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="13"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="12"/>
-      <c r="O30" s="12"/>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="11"/>
-      <c r="R30" s="12"/>
-      <c r="S30" s="12"/>
-      <c r="T30" s="13"/>
-      <c r="U30" s="11"/>
-      <c r="V30" s="12"/>
-      <c r="W30" s="12"/>
-      <c r="X30" s="13"/>
-      <c r="Y30" s="11"/>
-      <c r="Z30" s="12"/>
-      <c r="AA30" s="12"/>
-      <c r="AB30" s="13"/>
-      <c r="AC30" s="11"/>
-      <c r="AD30" s="12"/>
-      <c r="AE30" s="12"/>
-      <c r="AF30" s="13"/>
-      <c r="AG30" s="11"/>
-      <c r="AH30" s="12"/>
-      <c r="AI30" s="12"/>
-      <c r="AJ30" s="13"/>
-      <c r="AK30" s="11"/>
-      <c r="AL30" s="12"/>
-      <c r="AM30" s="12"/>
-      <c r="AN30" s="13"/>
-      <c r="AO30" s="11"/>
-      <c r="AP30" s="12"/>
-      <c r="AQ30" s="12"/>
-      <c r="AR30" s="13"/>
-      <c r="AS30" s="11"/>
-      <c r="AT30" s="12"/>
-      <c r="AU30" s="12"/>
-      <c r="AV30" s="13"/>
-      <c r="AW30" s="11"/>
-      <c r="AX30" s="12"/>
-      <c r="AY30" s="12"/>
-      <c r="AZ30" s="13"/>
-    </row>
-    <row r="31" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A31" s="43"/>
-      <c r="B31" s="39"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="49"/>
+      <c r="B30" s="80"/>
+      <c r="C30" s="81"/>
+      <c r="D30" s="82"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="9"/>
+      <c r="O30" s="9"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="9"/>
+      <c r="S30" s="9"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="8"/>
+      <c r="V30" s="9"/>
+      <c r="W30" s="9"/>
+      <c r="X30" s="10"/>
+      <c r="Y30" s="8"/>
+      <c r="Z30" s="9"/>
+      <c r="AA30" s="9"/>
+      <c r="AB30" s="10"/>
+      <c r="AC30" s="8"/>
+      <c r="AD30" s="9"/>
+      <c r="AE30" s="9"/>
+      <c r="AF30" s="10"/>
+      <c r="AG30" s="8"/>
+      <c r="AH30" s="9"/>
+      <c r="AI30" s="9"/>
+      <c r="AJ30" s="10"/>
+      <c r="AK30" s="8"/>
+      <c r="AL30" s="9"/>
+      <c r="AM30" s="9"/>
+      <c r="AN30" s="10"/>
+      <c r="AO30" s="8"/>
+      <c r="AP30" s="9"/>
+      <c r="AQ30" s="9"/>
+      <c r="AR30" s="10"/>
+      <c r="AS30" s="8"/>
+      <c r="AT30" s="9"/>
+      <c r="AU30" s="9"/>
+      <c r="AV30" s="10"/>
+      <c r="AW30" s="8"/>
+      <c r="AX30" s="9"/>
+      <c r="AY30" s="9"/>
+      <c r="AZ30" s="10"/>
+    </row>
+    <row r="31" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A31" s="62"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="51"/>
       <c r="E31" s="11"/>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
@@ -3101,11 +3111,11 @@
       <c r="AY31" s="12"/>
       <c r="AZ31" s="13"/>
     </row>
-    <row r="32" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A32" s="43"/>
-      <c r="B32" s="38"/>
-      <c r="C32" s="40"/>
-      <c r="D32" s="49"/>
+    <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="62"/>
+      <c r="B32" s="76"/>
+      <c r="C32" s="54"/>
+      <c r="D32" s="51"/>
       <c r="E32" s="11"/>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
@@ -3155,11 +3165,11 @@
       <c r="AY32" s="12"/>
       <c r="AZ32" s="13"/>
     </row>
-    <row r="33" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A33" s="43"/>
-      <c r="B33" s="39"/>
-      <c r="C33" s="40"/>
-      <c r="D33" s="49"/>
+    <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="62"/>
+      <c r="B33" s="72"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="51"/>
       <c r="E33" s="11"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
@@ -3209,11 +3219,11 @@
       <c r="AY33" s="12"/>
       <c r="AZ33" s="13"/>
     </row>
-    <row r="34" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A34" s="43"/>
-      <c r="B34" s="38"/>
-      <c r="C34" s="40"/>
-      <c r="D34" s="49"/>
+    <row r="34" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A34" s="62"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="79"/>
+      <c r="D34" s="51"/>
       <c r="E34" s="11"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
@@ -3263,11 +3273,11 @@
       <c r="AY34" s="12"/>
       <c r="AZ34" s="13"/>
     </row>
-    <row r="35" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A35" s="43"/>
-      <c r="B35" s="39"/>
-      <c r="C35" s="41"/>
-      <c r="D35" s="49"/>
+    <row r="35" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A35" s="62"/>
+      <c r="B35" s="72"/>
+      <c r="C35" s="79"/>
+      <c r="D35" s="51"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3317,13 +3327,11 @@
       <c r="AY35" s="12"/>
       <c r="AZ35" s="13"/>
     </row>
-    <row r="36" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A36" s="43"/>
-      <c r="B36" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="C36" s="41"/>
-      <c r="D36" s="49"/>
+    <row r="36" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A36" s="62"/>
+      <c r="B36" s="76"/>
+      <c r="C36" s="79"/>
+      <c r="D36" s="51"/>
       <c r="E36" s="11"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
@@ -3373,11 +3381,11 @@
       <c r="AY36" s="12"/>
       <c r="AZ36" s="13"/>
     </row>
-    <row r="37" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A37" s="43"/>
-      <c r="B37" s="59"/>
-      <c r="C37" s="41"/>
-      <c r="D37" s="49"/>
+    <row r="37" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A37" s="62"/>
+      <c r="B37" s="72"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="51"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3427,15 +3435,11 @@
       <c r="AY37" s="12"/>
       <c r="AZ37" s="13"/>
     </row>
-    <row r="38" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A38" s="43"/>
-      <c r="B38" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" s="41"/>
-      <c r="D38" s="49">
-        <v>0</v>
-      </c>
+    <row r="38" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A38" s="62"/>
+      <c r="B38" s="76"/>
+      <c r="C38" s="79"/>
+      <c r="D38" s="51"/>
       <c r="E38" s="11"/>
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
@@ -3485,11 +3489,11 @@
       <c r="AY38" s="12"/>
       <c r="AZ38" s="13"/>
     </row>
-    <row r="39" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="43"/>
-      <c r="B39" s="46"/>
-      <c r="C39" s="41"/>
-      <c r="D39" s="49"/>
+    <row r="39" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A39" s="62"/>
+      <c r="B39" s="72"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="51"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3539,69 +3543,67 @@
       <c r="AY39" s="12"/>
       <c r="AZ39" s="13"/>
     </row>
-    <row r="40" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A40" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="B40" s="45" t="s">
-        <v>24</v>
-      </c>
-      <c r="C40" s="47"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="9"/>
-      <c r="K40" s="9"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="8"/>
-      <c r="N40" s="9"/>
-      <c r="O40" s="9"/>
-      <c r="P40" s="10"/>
-      <c r="Q40" s="8"/>
-      <c r="R40" s="9"/>
-      <c r="S40" s="9"/>
-      <c r="T40" s="10"/>
-      <c r="U40" s="8"/>
-      <c r="V40" s="9"/>
-      <c r="W40" s="9"/>
-      <c r="X40" s="10"/>
-      <c r="Y40" s="8"/>
-      <c r="Z40" s="9"/>
-      <c r="AA40" s="9"/>
-      <c r="AB40" s="10"/>
-      <c r="AC40" s="8"/>
-      <c r="AD40" s="9"/>
-      <c r="AE40" s="9"/>
-      <c r="AF40" s="10"/>
-      <c r="AG40" s="8"/>
-      <c r="AH40" s="9"/>
-      <c r="AI40" s="9"/>
-      <c r="AJ40" s="10"/>
-      <c r="AK40" s="8"/>
-      <c r="AL40" s="9"/>
-      <c r="AM40" s="9"/>
-      <c r="AN40" s="10"/>
-      <c r="AO40" s="8"/>
-      <c r="AP40" s="9"/>
-      <c r="AQ40" s="9"/>
-      <c r="AR40" s="10"/>
-      <c r="AS40" s="8"/>
-      <c r="AT40" s="9"/>
-      <c r="AU40" s="9"/>
-      <c r="AV40" s="10"/>
-      <c r="AW40" s="8"/>
-      <c r="AX40" s="9"/>
-      <c r="AY40" s="9"/>
-      <c r="AZ40" s="10"/>
-    </row>
-    <row r="41" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A41" s="43"/>
-      <c r="B41" s="46"/>
-      <c r="C41" s="41"/>
-      <c r="D41" s="49"/>
+    <row r="40" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A40" s="62"/>
+      <c r="B40" s="78" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" s="54"/>
+      <c r="D40" s="51"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="12"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="11"/>
+      <c r="J40" s="12"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="13"/>
+      <c r="M40" s="11"/>
+      <c r="N40" s="12"/>
+      <c r="O40" s="12"/>
+      <c r="P40" s="13"/>
+      <c r="Q40" s="11"/>
+      <c r="R40" s="12"/>
+      <c r="S40" s="12"/>
+      <c r="T40" s="13"/>
+      <c r="U40" s="11"/>
+      <c r="V40" s="12"/>
+      <c r="W40" s="12"/>
+      <c r="X40" s="13"/>
+      <c r="Y40" s="11"/>
+      <c r="Z40" s="12"/>
+      <c r="AA40" s="12"/>
+      <c r="AB40" s="13"/>
+      <c r="AC40" s="11"/>
+      <c r="AD40" s="12"/>
+      <c r="AE40" s="12"/>
+      <c r="AF40" s="13"/>
+      <c r="AG40" s="11"/>
+      <c r="AH40" s="12"/>
+      <c r="AI40" s="12"/>
+      <c r="AJ40" s="13"/>
+      <c r="AK40" s="11"/>
+      <c r="AL40" s="12"/>
+      <c r="AM40" s="12"/>
+      <c r="AN40" s="13"/>
+      <c r="AO40" s="11"/>
+      <c r="AP40" s="12"/>
+      <c r="AQ40" s="12"/>
+      <c r="AR40" s="13"/>
+      <c r="AS40" s="11"/>
+      <c r="AT40" s="12"/>
+      <c r="AU40" s="12"/>
+      <c r="AV40" s="13"/>
+      <c r="AW40" s="11"/>
+      <c r="AX40" s="12"/>
+      <c r="AY40" s="12"/>
+      <c r="AZ40" s="13"/>
+    </row>
+    <row r="41" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A41" s="62"/>
+      <c r="B41" s="78"/>
+      <c r="C41" s="54"/>
+      <c r="D41" s="51"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3651,13 +3653,15 @@
       <c r="AY41" s="12"/>
       <c r="AZ41" s="13"/>
     </row>
-    <row r="42" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="43"/>
-      <c r="B42" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="C42" s="40"/>
-      <c r="D42" s="40"/>
+    <row r="42" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A42" s="62"/>
+      <c r="B42" s="52" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="54"/>
+      <c r="D42" s="51">
+        <v>0</v>
+      </c>
       <c r="E42" s="11"/>
       <c r="F42" s="12"/>
       <c r="G42" s="12"/>
@@ -3707,11 +3711,11 @@
       <c r="AY42" s="12"/>
       <c r="AZ42" s="13"/>
     </row>
-    <row r="43" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="43"/>
-      <c r="B43" s="39"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41"/>
+    <row r="43" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="62"/>
+      <c r="B43" s="52"/>
+      <c r="C43" s="54"/>
+      <c r="D43" s="51"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3761,125 +3765,125 @@
       <c r="AY43" s="12"/>
       <c r="AZ43" s="13"/>
     </row>
-    <row r="44" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="A44" s="43"/>
-      <c r="B44" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="C44" s="41"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="13"/>
-      <c r="I44" s="11"/>
-      <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
-      <c r="L44" s="13"/>
-      <c r="M44" s="11"/>
-      <c r="N44" s="12"/>
-      <c r="O44" s="12"/>
-      <c r="P44" s="13"/>
-      <c r="Q44" s="11"/>
-      <c r="R44" s="12"/>
-      <c r="S44" s="12"/>
-      <c r="T44" s="13"/>
-      <c r="U44" s="11"/>
-      <c r="V44" s="12"/>
-      <c r="W44" s="12"/>
-      <c r="X44" s="13"/>
-      <c r="Y44" s="11"/>
-      <c r="Z44" s="12"/>
-      <c r="AA44" s="12"/>
-      <c r="AB44" s="13"/>
-      <c r="AC44" s="11"/>
-      <c r="AD44" s="12"/>
-      <c r="AE44" s="12"/>
-      <c r="AF44" s="13"/>
-      <c r="AG44" s="11"/>
-      <c r="AH44" s="12"/>
-      <c r="AI44" s="12"/>
-      <c r="AJ44" s="13"/>
-      <c r="AK44" s="11"/>
-      <c r="AL44" s="12"/>
-      <c r="AM44" s="12"/>
-      <c r="AN44" s="13"/>
-      <c r="AO44" s="11"/>
-      <c r="AP44" s="12"/>
-      <c r="AQ44" s="12"/>
-      <c r="AR44" s="13"/>
-      <c r="AS44" s="11"/>
-      <c r="AT44" s="12"/>
-      <c r="AU44" s="12"/>
-      <c r="AV44" s="13"/>
-      <c r="AW44" s="11"/>
-      <c r="AX44" s="12"/>
-      <c r="AY44" s="12"/>
-      <c r="AZ44" s="13"/>
-    </row>
-    <row r="45" spans="1:52" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="44"/>
-      <c r="B45" s="50"/>
-      <c r="C45" s="51"/>
-      <c r="D45" s="52"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="18"/>
-      <c r="G45" s="18"/>
-      <c r="H45" s="19"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="18"/>
-      <c r="L45" s="19"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="18"/>
-      <c r="O45" s="18"/>
-      <c r="P45" s="19"/>
-      <c r="Q45" s="17"/>
-      <c r="R45" s="18"/>
-      <c r="S45" s="18"/>
-      <c r="T45" s="19"/>
-      <c r="U45" s="17"/>
-      <c r="V45" s="18"/>
-      <c r="W45" s="18"/>
-      <c r="X45" s="19"/>
-      <c r="Y45" s="17"/>
-      <c r="Z45" s="18"/>
-      <c r="AA45" s="18"/>
-      <c r="AB45" s="19"/>
-      <c r="AC45" s="17"/>
-      <c r="AD45" s="18"/>
-      <c r="AE45" s="18"/>
-      <c r="AF45" s="19"/>
-      <c r="AG45" s="17"/>
-      <c r="AH45" s="18"/>
-      <c r="AI45" s="18"/>
-      <c r="AJ45" s="19"/>
-      <c r="AK45" s="17"/>
-      <c r="AL45" s="18"/>
-      <c r="AM45" s="18"/>
-      <c r="AN45" s="19"/>
-      <c r="AO45" s="17"/>
-      <c r="AP45" s="18"/>
-      <c r="AQ45" s="18"/>
-      <c r="AR45" s="19"/>
-      <c r="AS45" s="17"/>
-      <c r="AT45" s="18"/>
-      <c r="AU45" s="18"/>
-      <c r="AV45" s="19"/>
-      <c r="AW45" s="17"/>
-      <c r="AX45" s="18"/>
-      <c r="AY45" s="18"/>
-      <c r="AZ45" s="19"/>
-    </row>
-    <row r="46" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="38" t="s">
-        <v>27</v>
-      </c>
-      <c r="C46" s="40"/>
-      <c r="D46" s="40"/>
+    <row r="44" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A44" s="61" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="80" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" s="81"/>
+      <c r="D44" s="82"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="8"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="8"/>
+      <c r="N44" s="9"/>
+      <c r="O44" s="9"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="8"/>
+      <c r="R44" s="9"/>
+      <c r="S44" s="9"/>
+      <c r="T44" s="10"/>
+      <c r="U44" s="8"/>
+      <c r="V44" s="9"/>
+      <c r="W44" s="9"/>
+      <c r="X44" s="10"/>
+      <c r="Y44" s="8"/>
+      <c r="Z44" s="9"/>
+      <c r="AA44" s="9"/>
+      <c r="AB44" s="10"/>
+      <c r="AC44" s="8"/>
+      <c r="AD44" s="9"/>
+      <c r="AE44" s="9"/>
+      <c r="AF44" s="10"/>
+      <c r="AG44" s="8"/>
+      <c r="AH44" s="9"/>
+      <c r="AI44" s="9"/>
+      <c r="AJ44" s="10"/>
+      <c r="AK44" s="8"/>
+      <c r="AL44" s="9"/>
+      <c r="AM44" s="9"/>
+      <c r="AN44" s="10"/>
+      <c r="AO44" s="8"/>
+      <c r="AP44" s="9"/>
+      <c r="AQ44" s="9"/>
+      <c r="AR44" s="10"/>
+      <c r="AS44" s="8"/>
+      <c r="AT44" s="9"/>
+      <c r="AU44" s="9"/>
+      <c r="AV44" s="10"/>
+      <c r="AW44" s="8"/>
+      <c r="AX44" s="9"/>
+      <c r="AY44" s="9"/>
+      <c r="AZ44" s="10"/>
+    </row>
+    <row r="45" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A45" s="62"/>
+      <c r="B45" s="52"/>
+      <c r="C45" s="54"/>
+      <c r="D45" s="51"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="13"/>
+      <c r="I45" s="11"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="13"/>
+      <c r="M45" s="11"/>
+      <c r="N45" s="12"/>
+      <c r="O45" s="12"/>
+      <c r="P45" s="13"/>
+      <c r="Q45" s="11"/>
+      <c r="R45" s="12"/>
+      <c r="S45" s="12"/>
+      <c r="T45" s="13"/>
+      <c r="U45" s="11"/>
+      <c r="V45" s="12"/>
+      <c r="W45" s="12"/>
+      <c r="X45" s="13"/>
+      <c r="Y45" s="11"/>
+      <c r="Z45" s="12"/>
+      <c r="AA45" s="12"/>
+      <c r="AB45" s="13"/>
+      <c r="AC45" s="11"/>
+      <c r="AD45" s="12"/>
+      <c r="AE45" s="12"/>
+      <c r="AF45" s="13"/>
+      <c r="AG45" s="11"/>
+      <c r="AH45" s="12"/>
+      <c r="AI45" s="12"/>
+      <c r="AJ45" s="13"/>
+      <c r="AK45" s="11"/>
+      <c r="AL45" s="12"/>
+      <c r="AM45" s="12"/>
+      <c r="AN45" s="13"/>
+      <c r="AO45" s="11"/>
+      <c r="AP45" s="12"/>
+      <c r="AQ45" s="12"/>
+      <c r="AR45" s="13"/>
+      <c r="AS45" s="11"/>
+      <c r="AT45" s="12"/>
+      <c r="AU45" s="12"/>
+      <c r="AV45" s="13"/>
+      <c r="AW45" s="11"/>
+      <c r="AX45" s="12"/>
+      <c r="AY45" s="12"/>
+      <c r="AZ45" s="13"/>
+    </row>
+    <row r="46" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="62"/>
+      <c r="B46" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="C46" s="79"/>
+      <c r="D46" s="79"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -3929,11 +3933,11 @@
       <c r="AY46" s="12"/>
       <c r="AZ46" s="13"/>
     </row>
-    <row r="47" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="43"/>
-      <c r="B47" s="39"/>
-      <c r="C47" s="41"/>
-      <c r="D47" s="41"/>
+    <row r="47" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="62"/>
+      <c r="B47" s="72"/>
+      <c r="C47" s="54"/>
+      <c r="D47" s="54"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -3983,15 +3987,13 @@
       <c r="AY47" s="12"/>
       <c r="AZ47" s="13"/>
     </row>
-    <row r="48" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="43"/>
-      <c r="B48" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="C48" s="40"/>
-      <c r="D48" s="40">
-        <v>0</v>
-      </c>
+    <row r="48" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A48" s="62"/>
+      <c r="B48" s="52" t="s">
+        <v>24</v>
+      </c>
+      <c r="C48" s="54"/>
+      <c r="D48" s="51"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4041,11 +4043,11 @@
       <c r="AY48" s="12"/>
       <c r="AZ48" s="13"/>
     </row>
-    <row r="49" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="44"/>
-      <c r="B49" s="53"/>
-      <c r="C49" s="41"/>
-      <c r="D49" s="41"/>
+    <row r="49" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="63"/>
+      <c r="B49" s="73"/>
+      <c r="C49" s="74"/>
+      <c r="D49" s="75"/>
       <c r="E49" s="17"/>
       <c r="F49" s="18"/>
       <c r="G49" s="18"/>
@@ -4095,72 +4097,380 @@
       <c r="AY49" s="18"/>
       <c r="AZ49" s="19"/>
     </row>
-    <row r="50" spans="1:52" x14ac:dyDescent="0.3">
-      <c r="B50" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C50" s="5">
-        <f>SUM(C4:C49)</f>
+    <row r="50" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="61" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="76" t="s">
+        <v>25</v>
+      </c>
+      <c r="C50" s="79"/>
+      <c r="D50" s="79"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="13"/>
+      <c r="I50" s="11"/>
+      <c r="J50" s="12"/>
+      <c r="K50" s="12"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="11"/>
+      <c r="N50" s="12"/>
+      <c r="O50" s="12"/>
+      <c r="P50" s="13"/>
+      <c r="Q50" s="11"/>
+      <c r="R50" s="12"/>
+      <c r="S50" s="12"/>
+      <c r="T50" s="13"/>
+      <c r="U50" s="11"/>
+      <c r="V50" s="12"/>
+      <c r="W50" s="12"/>
+      <c r="X50" s="13"/>
+      <c r="Y50" s="11"/>
+      <c r="Z50" s="12"/>
+      <c r="AA50" s="12"/>
+      <c r="AB50" s="13"/>
+      <c r="AC50" s="11"/>
+      <c r="AD50" s="12"/>
+      <c r="AE50" s="12"/>
+      <c r="AF50" s="13"/>
+      <c r="AG50" s="11"/>
+      <c r="AH50" s="12"/>
+      <c r="AI50" s="12"/>
+      <c r="AJ50" s="13"/>
+      <c r="AK50" s="11"/>
+      <c r="AL50" s="12"/>
+      <c r="AM50" s="12"/>
+      <c r="AN50" s="13"/>
+      <c r="AO50" s="11"/>
+      <c r="AP50" s="12"/>
+      <c r="AQ50" s="12"/>
+      <c r="AR50" s="13"/>
+      <c r="AS50" s="11"/>
+      <c r="AT50" s="12"/>
+      <c r="AU50" s="12"/>
+      <c r="AV50" s="13"/>
+      <c r="AW50" s="11"/>
+      <c r="AX50" s="12"/>
+      <c r="AY50" s="12"/>
+      <c r="AZ50" s="13"/>
+    </row>
+    <row r="51" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="62"/>
+      <c r="B51" s="72"/>
+      <c r="C51" s="54"/>
+      <c r="D51" s="54"/>
+      <c r="E51" s="11"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="12"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="12"/>
+      <c r="K51" s="12"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="11"/>
+      <c r="N51" s="12"/>
+      <c r="O51" s="12"/>
+      <c r="P51" s="13"/>
+      <c r="Q51" s="11"/>
+      <c r="R51" s="12"/>
+      <c r="S51" s="12"/>
+      <c r="T51" s="13"/>
+      <c r="U51" s="11"/>
+      <c r="V51" s="12"/>
+      <c r="W51" s="12"/>
+      <c r="X51" s="13"/>
+      <c r="Y51" s="11"/>
+      <c r="Z51" s="12"/>
+      <c r="AA51" s="12"/>
+      <c r="AB51" s="13"/>
+      <c r="AC51" s="11"/>
+      <c r="AD51" s="12"/>
+      <c r="AE51" s="12"/>
+      <c r="AF51" s="13"/>
+      <c r="AG51" s="11"/>
+      <c r="AH51" s="12"/>
+      <c r="AI51" s="12"/>
+      <c r="AJ51" s="13"/>
+      <c r="AK51" s="11"/>
+      <c r="AL51" s="12"/>
+      <c r="AM51" s="12"/>
+      <c r="AN51" s="13"/>
+      <c r="AO51" s="11"/>
+      <c r="AP51" s="12"/>
+      <c r="AQ51" s="12"/>
+      <c r="AR51" s="13"/>
+      <c r="AS51" s="11"/>
+      <c r="AT51" s="12"/>
+      <c r="AU51" s="12"/>
+      <c r="AV51" s="13"/>
+      <c r="AW51" s="11"/>
+      <c r="AX51" s="12"/>
+      <c r="AY51" s="12"/>
+      <c r="AZ51" s="13"/>
+    </row>
+    <row r="52" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="62"/>
+      <c r="B52" s="76" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="79"/>
+      <c r="D52" s="79">
         <v>0</v>
       </c>
-      <c r="D50" s="5">
-        <f>SUM(D4:D49)</f>
+      <c r="E52" s="11"/>
+      <c r="F52" s="12"/>
+      <c r="G52" s="12"/>
+      <c r="H52" s="13"/>
+      <c r="I52" s="11"/>
+      <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="13"/>
+      <c r="M52" s="11"/>
+      <c r="N52" s="12"/>
+      <c r="O52" s="12"/>
+      <c r="P52" s="13"/>
+      <c r="Q52" s="11"/>
+      <c r="R52" s="12"/>
+      <c r="S52" s="12"/>
+      <c r="T52" s="13"/>
+      <c r="U52" s="11"/>
+      <c r="V52" s="12"/>
+      <c r="W52" s="12"/>
+      <c r="X52" s="13"/>
+      <c r="Y52" s="11"/>
+      <c r="Z52" s="12"/>
+      <c r="AA52" s="12"/>
+      <c r="AB52" s="13"/>
+      <c r="AC52" s="11"/>
+      <c r="AD52" s="12"/>
+      <c r="AE52" s="12"/>
+      <c r="AF52" s="13"/>
+      <c r="AG52" s="11"/>
+      <c r="AH52" s="12"/>
+      <c r="AI52" s="12"/>
+      <c r="AJ52" s="13"/>
+      <c r="AK52" s="11"/>
+      <c r="AL52" s="12"/>
+      <c r="AM52" s="12"/>
+      <c r="AN52" s="13"/>
+      <c r="AO52" s="11"/>
+      <c r="AP52" s="12"/>
+      <c r="AQ52" s="12"/>
+      <c r="AR52" s="13"/>
+      <c r="AS52" s="11"/>
+      <c r="AT52" s="12"/>
+      <c r="AU52" s="12"/>
+      <c r="AV52" s="13"/>
+      <c r="AW52" s="11"/>
+      <c r="AX52" s="12"/>
+      <c r="AY52" s="12"/>
+      <c r="AZ52" s="13"/>
+    </row>
+    <row r="53" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="63"/>
+      <c r="B53" s="84"/>
+      <c r="C53" s="54"/>
+      <c r="D53" s="54"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="19"/>
+      <c r="I53" s="17"/>
+      <c r="J53" s="18"/>
+      <c r="K53" s="18"/>
+      <c r="L53" s="19"/>
+      <c r="M53" s="17"/>
+      <c r="N53" s="18"/>
+      <c r="O53" s="18"/>
+      <c r="P53" s="19"/>
+      <c r="Q53" s="17"/>
+      <c r="R53" s="18"/>
+      <c r="S53" s="18"/>
+      <c r="T53" s="19"/>
+      <c r="U53" s="17"/>
+      <c r="V53" s="18"/>
+      <c r="W53" s="18"/>
+      <c r="X53" s="19"/>
+      <c r="Y53" s="17"/>
+      <c r="Z53" s="18"/>
+      <c r="AA53" s="18"/>
+      <c r="AB53" s="19"/>
+      <c r="AC53" s="17"/>
+      <c r="AD53" s="18"/>
+      <c r="AE53" s="18"/>
+      <c r="AF53" s="19"/>
+      <c r="AG53" s="17"/>
+      <c r="AH53" s="18"/>
+      <c r="AI53" s="18"/>
+      <c r="AJ53" s="19"/>
+      <c r="AK53" s="17"/>
+      <c r="AL53" s="18"/>
+      <c r="AM53" s="18"/>
+      <c r="AN53" s="19"/>
+      <c r="AO53" s="17"/>
+      <c r="AP53" s="18"/>
+      <c r="AQ53" s="18"/>
+      <c r="AR53" s="19"/>
+      <c r="AS53" s="17"/>
+      <c r="AT53" s="18"/>
+      <c r="AU53" s="18"/>
+      <c r="AV53" s="19"/>
+      <c r="AW53" s="17"/>
+      <c r="AX53" s="18"/>
+      <c r="AY53" s="18"/>
+      <c r="AZ53" s="19"/>
+    </row>
+    <row r="54" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C54" s="5">
+        <f>SUM(C4:C53)</f>
         <v>0</v>
       </c>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="6"/>
-      <c r="N50" s="6"/>
-      <c r="O50" s="6"/>
-      <c r="P50" s="6"/>
-      <c r="Q50" s="6"/>
-      <c r="R50" s="6"/>
-      <c r="S50" s="6"/>
-      <c r="T50" s="6"/>
-      <c r="U50" s="6"/>
-      <c r="V50" s="6"/>
-      <c r="W50" s="6"/>
-      <c r="X50" s="6"/>
-      <c r="Y50" s="6"/>
-      <c r="Z50" s="6"/>
-      <c r="AA50" s="6"/>
-      <c r="AB50" s="6"/>
-      <c r="AC50" s="6"/>
-      <c r="AD50" s="6"/>
-      <c r="AE50" s="6"/>
-      <c r="AF50" s="6"/>
-      <c r="AG50" s="6"/>
-      <c r="AH50" s="6"/>
-      <c r="AI50" s="6"/>
-      <c r="AJ50" s="6"/>
-      <c r="AK50" s="6"/>
-      <c r="AL50" s="6"/>
-      <c r="AM50" s="6"/>
-      <c r="AN50" s="6"/>
-      <c r="AO50" s="6"/>
-      <c r="AP50" s="6"/>
-      <c r="AQ50" s="6"/>
-      <c r="AR50" s="6"/>
-      <c r="AS50" s="6"/>
-      <c r="AT50" s="6"/>
-      <c r="AU50" s="6"/>
-      <c r="AV50" s="6"/>
-      <c r="AW50" s="6"/>
-      <c r="AX50" s="6"/>
-      <c r="AY50" s="7"/>
-      <c r="AZ50" s="7"/>
-    </row>
-    <row r="51" spans="1:52" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="D54" s="5">
+        <f>SUM(D4:D53)</f>
+        <v>0</v>
+      </c>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="6"/>
+      <c r="N54" s="6"/>
+      <c r="O54" s="6"/>
+      <c r="P54" s="6"/>
+      <c r="Q54" s="6"/>
+      <c r="R54" s="6"/>
+      <c r="S54" s="6"/>
+      <c r="T54" s="6"/>
+      <c r="U54" s="6"/>
+      <c r="V54" s="6"/>
+      <c r="W54" s="6"/>
+      <c r="X54" s="6"/>
+      <c r="Y54" s="6"/>
+      <c r="Z54" s="6"/>
+      <c r="AA54" s="6"/>
+      <c r="AB54" s="6"/>
+      <c r="AC54" s="6"/>
+      <c r="AD54" s="6"/>
+      <c r="AE54" s="6"/>
+      <c r="AF54" s="6"/>
+      <c r="AG54" s="6"/>
+      <c r="AH54" s="6"/>
+      <c r="AI54" s="6"/>
+      <c r="AJ54" s="6"/>
+      <c r="AK54" s="6"/>
+      <c r="AL54" s="6"/>
+      <c r="AM54" s="6"/>
+      <c r="AN54" s="6"/>
+      <c r="AO54" s="6"/>
+      <c r="AP54" s="6"/>
+      <c r="AQ54" s="6"/>
+      <c r="AR54" s="6"/>
+      <c r="AS54" s="6"/>
+      <c r="AT54" s="6"/>
+      <c r="AU54" s="6"/>
+      <c r="AV54" s="6"/>
+      <c r="AW54" s="6"/>
+      <c r="AX54" s="6"/>
+      <c r="AY54" s="7"/>
+      <c r="AZ54" s="7"/>
+    </row>
+    <row r="55" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="102">
+  <mergeCells count="108">
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A43"/>
+    <mergeCell ref="A44:A49"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="C42:C43"/>
     <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="D36:D37"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
@@ -4168,8 +4478,8 @@
     <mergeCell ref="AW2:AZ2"/>
     <mergeCell ref="AS1:AV1"/>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="A14:A23"/>
+    <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A18:A27"/>
     <mergeCell ref="AK1:AN1"/>
     <mergeCell ref="AO1:AR1"/>
     <mergeCell ref="E1:H1"/>
@@ -4183,84 +4493,6 @@
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="U2:X2"/>
     <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A26:A39"/>
-    <mergeCell ref="A40:A45"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Doku, CSS für Home Page und Readme aktualisiert
</commit_message>
<xml_diff>
--- a/pa_zeitplan_vorlage.xlsx
+++ b/pa_zeitplan_vorlage.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E91C9B9C-0087-4900-9FCF-4B02E68C6C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6844E8F4-C01D-4C39-8D3A-2F3B11743ABC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
   <si>
     <t>IPERKA Phase</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Systembeschreibung, Kurzfassung, Anleitutungm Glossar, etc. erstellen</t>
   </si>
   <si>
-    <t>10min</t>
-  </si>
-  <si>
     <t>Montag</t>
   </si>
   <si>
@@ -133,13 +130,13 @@
     <t>Freitag</t>
   </si>
   <si>
-    <t>1h</t>
+    <t>User Storys aufschreiben</t>
   </si>
   <si>
-    <t>1h 30min</t>
+    <t>Weitere Features überlegen die nützlich sein könnten</t>
   </si>
   <si>
-    <t>User Storys aufschreiben</t>
+    <t>0.333333</t>
   </si>
 </sst>
 </file>
@@ -802,6 +799,87 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -811,17 +889,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -832,6 +901,33 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -840,105 +936,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1274,162 +1271,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="69"/>
-      <c r="E1" s="48" t="s">
+      <c r="D1" s="86"/>
+      <c r="E1" s="75" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="48" t="s">
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="48" t="s">
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="48" t="s">
+      <c r="R1" s="76"/>
+      <c r="S1" s="76"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="R1" s="49"/>
-      <c r="S1" s="49"/>
-      <c r="T1" s="50"/>
-      <c r="U1" s="48" t="s">
-        <v>32</v>
-      </c>
-      <c r="V1" s="49"/>
-      <c r="W1" s="49"/>
-      <c r="X1" s="50"/>
-      <c r="Y1" s="48" t="s">
+      <c r="V1" s="76"/>
+      <c r="W1" s="76"/>
+      <c r="X1" s="77"/>
+      <c r="Y1" s="75" t="s">
+        <v>28</v>
+      </c>
+      <c r="Z1" s="76"/>
+      <c r="AA1" s="76"/>
+      <c r="AB1" s="77"/>
+      <c r="AC1" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="Z1" s="49"/>
-      <c r="AA1" s="49"/>
-      <c r="AB1" s="50"/>
-      <c r="AC1" s="48" t="s">
+      <c r="AD1" s="76"/>
+      <c r="AE1" s="76"/>
+      <c r="AF1" s="77"/>
+      <c r="AG1" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="AD1" s="49"/>
-      <c r="AE1" s="49"/>
-      <c r="AF1" s="50"/>
-      <c r="AG1" s="48" t="s">
+      <c r="AH1" s="76"/>
+      <c r="AI1" s="76"/>
+      <c r="AJ1" s="77"/>
+      <c r="AK1" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="49"/>
-      <c r="AI1" s="49"/>
-      <c r="AJ1" s="50"/>
-      <c r="AK1" s="48" t="s">
-        <v>32</v>
-      </c>
-      <c r="AL1" s="49"/>
-      <c r="AM1" s="49"/>
-      <c r="AN1" s="50"/>
-      <c r="AO1" s="48" t="s">
-        <v>28</v>
-      </c>
-      <c r="AP1" s="49"/>
-      <c r="AQ1" s="49"/>
-      <c r="AR1" s="50"/>
-      <c r="AS1" s="48"/>
-      <c r="AT1" s="49"/>
-      <c r="AU1" s="49"/>
-      <c r="AV1" s="50"/>
-      <c r="AW1" s="48"/>
-      <c r="AX1" s="49"/>
-      <c r="AY1" s="49"/>
-      <c r="AZ1" s="50"/>
+      <c r="AL1" s="76"/>
+      <c r="AM1" s="76"/>
+      <c r="AN1" s="77"/>
+      <c r="AO1" s="75" t="s">
+        <v>27</v>
+      </c>
+      <c r="AP1" s="76"/>
+      <c r="AQ1" s="76"/>
+      <c r="AR1" s="77"/>
+      <c r="AS1" s="75"/>
+      <c r="AT1" s="76"/>
+      <c r="AU1" s="76"/>
+      <c r="AV1" s="77"/>
+      <c r="AW1" s="75"/>
+      <c r="AX1" s="76"/>
+      <c r="AY1" s="76"/>
+      <c r="AZ1" s="77"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="59"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="55">
+      <c r="A2" s="92"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="79">
         <v>44781</v>
       </c>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="55">
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="79">
         <v>44782</v>
       </c>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="55">
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="79">
         <v>44783</v>
       </c>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="57"/>
-      <c r="Q2" s="55">
+      <c r="N2" s="80"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="81"/>
+      <c r="Q2" s="79">
         <v>44784</v>
       </c>
-      <c r="R2" s="56"/>
-      <c r="S2" s="56"/>
-      <c r="T2" s="57"/>
-      <c r="U2" s="55">
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="79">
         <v>44785</v>
       </c>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="57"/>
-      <c r="Y2" s="55">
+      <c r="V2" s="80"/>
+      <c r="W2" s="80"/>
+      <c r="X2" s="81"/>
+      <c r="Y2" s="79">
         <v>44789</v>
       </c>
-      <c r="Z2" s="56"/>
-      <c r="AA2" s="56"/>
-      <c r="AB2" s="57"/>
-      <c r="AC2" s="55">
+      <c r="Z2" s="80"/>
+      <c r="AA2" s="80"/>
+      <c r="AB2" s="81"/>
+      <c r="AC2" s="79">
         <v>44790</v>
       </c>
-      <c r="AD2" s="56"/>
-      <c r="AE2" s="56"/>
-      <c r="AF2" s="57"/>
-      <c r="AG2" s="55">
+      <c r="AD2" s="80"/>
+      <c r="AE2" s="80"/>
+      <c r="AF2" s="81"/>
+      <c r="AG2" s="79">
         <v>44791</v>
       </c>
-      <c r="AH2" s="56"/>
-      <c r="AI2" s="56"/>
-      <c r="AJ2" s="57"/>
-      <c r="AK2" s="55">
+      <c r="AH2" s="80"/>
+      <c r="AI2" s="80"/>
+      <c r="AJ2" s="81"/>
+      <c r="AK2" s="79">
         <v>44792</v>
       </c>
-      <c r="AL2" s="56"/>
-      <c r="AM2" s="56"/>
-      <c r="AN2" s="57"/>
-      <c r="AO2" s="55">
+      <c r="AL2" s="80"/>
+      <c r="AM2" s="80"/>
+      <c r="AN2" s="81"/>
+      <c r="AO2" s="79">
         <v>44795</v>
       </c>
-      <c r="AP2" s="56"/>
-      <c r="AQ2" s="56"/>
-      <c r="AR2" s="57"/>
-      <c r="AS2" s="55"/>
-      <c r="AT2" s="56"/>
-      <c r="AU2" s="56"/>
-      <c r="AV2" s="57"/>
-      <c r="AW2" s="55"/>
-      <c r="AX2" s="56"/>
-      <c r="AY2" s="56"/>
-      <c r="AZ2" s="57"/>
+      <c r="AP2" s="80"/>
+      <c r="AQ2" s="80"/>
+      <c r="AR2" s="81"/>
+      <c r="AS2" s="79"/>
+      <c r="AT2" s="80"/>
+      <c r="AU2" s="80"/>
+      <c r="AV2" s="81"/>
+      <c r="AW2" s="79"/>
+      <c r="AX2" s="80"/>
+      <c r="AY2" s="80"/>
+      <c r="AZ2" s="81"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="60"/>
-      <c r="B3" s="67"/>
+      <c r="A3" s="93"/>
+      <c r="B3" s="84"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1567,11 +1564,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="72" t="s">
+      <c r="B4" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="53"/>
-      <c r="D4" s="87"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="67"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1627,9 +1624,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="86"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="85"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="68"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1685,9 +1682,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="78"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="51"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="59"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1732,9 +1729,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="76"/>
-      <c r="C7" s="64"/>
-      <c r="D7" s="85"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="68"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1789,17 +1786,17 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="80" t="s">
+      <c r="B8" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="81" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="91" t="s">
-        <v>27</v>
+      <c r="C8" s="57">
+        <v>0.1</v>
+      </c>
+      <c r="D8" s="73">
+        <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
       <c r="F8" s="47"/>
@@ -1855,10 +1852,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="62"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="92"/>
+      <c r="A9" s="53"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="74"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1909,15 +1906,15 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="62"/>
-      <c r="B10" s="52" t="s">
+      <c r="A10" s="53"/>
+      <c r="B10" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="53" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="53" t="s">
-        <v>34</v>
+      <c r="C10" s="65">
+        <v>1</v>
+      </c>
+      <c r="D10" s="65">
+        <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
       <c r="F10" s="43"/>
@@ -1969,10 +1966,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="62"/>
-      <c r="B11" s="52"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
+      <c r="A11" s="53"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="51"/>
+      <c r="D11" s="51"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2023,12 +2020,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="62"/>
-      <c r="B12" s="52" t="s">
+      <c r="A12" s="53"/>
+      <c r="B12" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2079,10 +2076,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62"/>
-      <c r="B13" s="52"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
+      <c r="A13" s="53"/>
+      <c r="B13" s="56"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="51"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2133,12 +2130,16 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="62"/>
-      <c r="B14" s="52" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
+      <c r="A14" s="53"/>
+      <c r="B14" s="56" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="65" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="65" t="s">
+        <v>34</v>
+      </c>
       <c r="E14" s="42"/>
       <c r="F14" s="43"/>
       <c r="G14" s="43"/>
@@ -2189,10 +2190,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="62"/>
-      <c r="B15" s="52"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
+      <c r="A15" s="53"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2243,10 +2244,16 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="62"/>
-      <c r="B16" s="86"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="51"/>
+      <c r="A16" s="53"/>
+      <c r="B16" s="64" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="51" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="59" t="s">
+        <v>34</v>
+      </c>
       <c r="E16" s="20"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -2297,10 +2304,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63"/>
-      <c r="B17" s="93"/>
-      <c r="C17" s="74"/>
-      <c r="D17" s="75"/>
+      <c r="A17" s="54"/>
+      <c r="B17" s="89"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="62"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2351,14 +2358,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="61" t="s">
+      <c r="A18" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="83" t="s">
+      <c r="B18" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="81"/>
-      <c r="D18" s="82"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="58"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2409,10 +2416,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="62"/>
-      <c r="B19" s="84"/>
-      <c r="C19" s="54"/>
-      <c r="D19" s="51"/>
+      <c r="A19" s="53"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="59"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2463,12 +2470,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="62"/>
-      <c r="B20" s="52" t="s">
+      <c r="A20" s="53"/>
+      <c r="B20" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="51"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="59"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2508,10 +2515,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="62"/>
-      <c r="B21" s="52"/>
-      <c r="C21" s="54"/>
-      <c r="D21" s="51"/>
+      <c r="A21" s="53"/>
+      <c r="B21" s="56"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="59"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2562,10 +2569,10 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="62"/>
-      <c r="B22" s="52"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="51"/>
+      <c r="A22" s="53"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="51"/>
+      <c r="D22" s="59"/>
       <c r="E22" s="11"/>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
@@ -2616,10 +2623,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="62"/>
-      <c r="B23" s="52"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="51"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="59"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2670,10 +2677,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="62"/>
-      <c r="B24" s="86"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="88"/>
+      <c r="A24" s="53"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="70"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2724,10 +2731,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="62"/>
-      <c r="B25" s="72"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="89"/>
+      <c r="A25" s="53"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="65"/>
+      <c r="D25" s="71"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2778,12 +2785,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="62"/>
-      <c r="B26" s="52" t="s">
+      <c r="A26" s="53"/>
+      <c r="B26" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="64"/>
-      <c r="D26" s="88">
+      <c r="C26" s="66"/>
+      <c r="D26" s="70">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2836,10 +2843,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="63"/>
-      <c r="B27" s="52"/>
-      <c r="C27" s="77"/>
-      <c r="D27" s="90"/>
+      <c r="A27" s="54"/>
+      <c r="B27" s="56"/>
+      <c r="C27" s="90"/>
+      <c r="D27" s="72"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2890,14 +2897,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="61" t="s">
+      <c r="A28" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="80" t="s">
+      <c r="B28" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="81"/>
-      <c r="D28" s="82"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="58"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2948,10 +2955,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="62"/>
-      <c r="B29" s="73"/>
-      <c r="C29" s="74"/>
-      <c r="D29" s="75"/>
+      <c r="A29" s="53"/>
+      <c r="B29" s="60"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="62"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3002,12 +3009,12 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="61" t="s">
+      <c r="A30" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="80"/>
-      <c r="C30" s="81"/>
-      <c r="D30" s="82"/>
+      <c r="B30" s="55"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="58"/>
       <c r="E30" s="8"/>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -3058,10 +3065,10 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="62"/>
-      <c r="B31" s="52"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="51"/>
+      <c r="A31" s="53"/>
+      <c r="B31" s="56"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="59"/>
       <c r="E31" s="11"/>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
@@ -3112,10 +3119,10 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="62"/>
-      <c r="B32" s="76"/>
-      <c r="C32" s="54"/>
-      <c r="D32" s="51"/>
+      <c r="A32" s="53"/>
+      <c r="B32" s="48"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="59"/>
       <c r="E32" s="11"/>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
@@ -3166,10 +3173,10 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="62"/>
-      <c r="B33" s="72"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="51"/>
+      <c r="A33" s="53"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="59"/>
       <c r="E33" s="11"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
@@ -3220,10 +3227,10 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A34" s="62"/>
-      <c r="B34" s="76"/>
-      <c r="C34" s="79"/>
-      <c r="D34" s="51"/>
+      <c r="A34" s="53"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="50"/>
+      <c r="D34" s="59"/>
       <c r="E34" s="11"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
@@ -3274,10 +3281,10 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A35" s="62"/>
-      <c r="B35" s="72"/>
-      <c r="C35" s="79"/>
-      <c r="D35" s="51"/>
+      <c r="A35" s="53"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="50"/>
+      <c r="D35" s="59"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3328,10 +3335,10 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A36" s="62"/>
-      <c r="B36" s="76"/>
-      <c r="C36" s="79"/>
-      <c r="D36" s="51"/>
+      <c r="A36" s="53"/>
+      <c r="B36" s="48"/>
+      <c r="C36" s="50"/>
+      <c r="D36" s="59"/>
       <c r="E36" s="11"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
@@ -3382,10 +3389,10 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A37" s="62"/>
-      <c r="B37" s="72"/>
-      <c r="C37" s="79"/>
-      <c r="D37" s="51"/>
+      <c r="A37" s="53"/>
+      <c r="B37" s="49"/>
+      <c r="C37" s="50"/>
+      <c r="D37" s="59"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3436,10 +3443,10 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A38" s="62"/>
-      <c r="B38" s="76"/>
-      <c r="C38" s="79"/>
-      <c r="D38" s="51"/>
+      <c r="A38" s="53"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="50"/>
+      <c r="D38" s="59"/>
       <c r="E38" s="11"/>
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
@@ -3490,10 +3497,10 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A39" s="62"/>
-      <c r="B39" s="72"/>
-      <c r="C39" s="54"/>
-      <c r="D39" s="51"/>
+      <c r="A39" s="53"/>
+      <c r="B39" s="49"/>
+      <c r="C39" s="51"/>
+      <c r="D39" s="59"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3544,12 +3551,12 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A40" s="62"/>
-      <c r="B40" s="78" t="s">
+      <c r="A40" s="53"/>
+      <c r="B40" s="69" t="s">
         <v>26</v>
       </c>
-      <c r="C40" s="54"/>
-      <c r="D40" s="51"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="59"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -3600,10 +3607,10 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A41" s="62"/>
-      <c r="B41" s="78"/>
-      <c r="C41" s="54"/>
-      <c r="D41" s="51"/>
+      <c r="A41" s="53"/>
+      <c r="B41" s="69"/>
+      <c r="C41" s="51"/>
+      <c r="D41" s="59"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3654,12 +3661,12 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="62"/>
-      <c r="B42" s="52" t="s">
+      <c r="A42" s="53"/>
+      <c r="B42" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="C42" s="54"/>
-      <c r="D42" s="51">
+      <c r="C42" s="51"/>
+      <c r="D42" s="59">
         <v>0</v>
       </c>
       <c r="E42" s="11"/>
@@ -3712,10 +3719,10 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="62"/>
-      <c r="B43" s="52"/>
-      <c r="C43" s="54"/>
-      <c r="D43" s="51"/>
+      <c r="A43" s="53"/>
+      <c r="B43" s="56"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="59"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3766,14 +3773,14 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A44" s="61" t="s">
+      <c r="A44" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="B44" s="80" t="s">
+      <c r="B44" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="C44" s="81"/>
-      <c r="D44" s="82"/>
+      <c r="C44" s="57"/>
+      <c r="D44" s="58"/>
       <c r="E44" s="8"/>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -3824,10 +3831,10 @@
       <c r="AZ44" s="10"/>
     </row>
     <row r="45" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A45" s="62"/>
-      <c r="B45" s="52"/>
-      <c r="C45" s="54"/>
-      <c r="D45" s="51"/>
+      <c r="A45" s="53"/>
+      <c r="B45" s="56"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="59"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -3878,12 +3885,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="62"/>
-      <c r="B46" s="76" t="s">
+      <c r="A46" s="53"/>
+      <c r="B46" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="C46" s="79"/>
-      <c r="D46" s="79"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="50"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -3934,10 +3941,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="62"/>
-      <c r="B47" s="72"/>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
+      <c r="A47" s="53"/>
+      <c r="B47" s="49"/>
+      <c r="C47" s="51"/>
+      <c r="D47" s="51"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -3988,12 +3995,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="62"/>
-      <c r="B48" s="52" t="s">
+      <c r="A48" s="53"/>
+      <c r="B48" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="C48" s="54"/>
-      <c r="D48" s="51"/>
+      <c r="C48" s="51"/>
+      <c r="D48" s="59"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4044,10 +4051,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="63"/>
-      <c r="B49" s="73"/>
-      <c r="C49" s="74"/>
-      <c r="D49" s="75"/>
+      <c r="A49" s="54"/>
+      <c r="B49" s="60"/>
+      <c r="C49" s="61"/>
+      <c r="D49" s="62"/>
       <c r="E49" s="17"/>
       <c r="F49" s="18"/>
       <c r="G49" s="18"/>
@@ -4098,14 +4105,14 @@
       <c r="AZ49" s="19"/>
     </row>
     <row r="50" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="61" t="s">
+      <c r="A50" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="B50" s="76" t="s">
+      <c r="B50" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="C50" s="79"/>
-      <c r="D50" s="79"/>
+      <c r="C50" s="50"/>
+      <c r="D50" s="50"/>
       <c r="E50" s="11"/>
       <c r="F50" s="12"/>
       <c r="G50" s="12"/>
@@ -4156,10 +4163,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="62"/>
-      <c r="B51" s="72"/>
-      <c r="C51" s="54"/>
-      <c r="D51" s="54"/>
+      <c r="A51" s="53"/>
+      <c r="B51" s="49"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="51"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4210,12 +4217,12 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="62"/>
-      <c r="B52" s="76" t="s">
+      <c r="A52" s="53"/>
+      <c r="B52" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="C52" s="79"/>
-      <c r="D52" s="79">
+      <c r="C52" s="50"/>
+      <c r="D52" s="50">
         <v>0</v>
       </c>
       <c r="E52" s="11"/>
@@ -4268,10 +4275,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="63"/>
-      <c r="B53" s="84"/>
-      <c r="C53" s="54"/>
-      <c r="D53" s="54"/>
+      <c r="A53" s="54"/>
+      <c r="B53" s="63"/>
+      <c r="C53" s="51"/>
+      <c r="D53" s="51"/>
       <c r="E53" s="17"/>
       <c r="F53" s="18"/>
       <c r="G53" s="18"/>
@@ -4327,11 +4334,11 @@
       </c>
       <c r="C54" s="5">
         <f>SUM(C4:C53)</f>
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="D54" s="5">
         <f>SUM(D4:D53)</f>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
@@ -4385,42 +4392,54 @@
     <row r="55" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="108">
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="AW2:AZ2"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="AK1:AN1"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="AK2:AN2"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A43"/>
+    <mergeCell ref="A44:A49"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="C42:C43"/>
     <mergeCell ref="C36:C37"/>
     <mergeCell ref="B38:B39"/>
     <mergeCell ref="C38:C39"/>
@@ -4445,54 +4464,42 @@
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="B8:B9"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A43"/>
-    <mergeCell ref="A44:A49"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="AW2:AZ2"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A8:A17"/>
-    <mergeCell ref="A18:A27"/>
-    <mergeCell ref="AK1:AN1"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="AK2:AN2"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="D52:D53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>